<commit_message>
Sync BD docs 2026-07-08-v1 (202607160645) from my-cloud-project@a046d9b
</commit_message>
<xml_diff>
--- a/瓶与井世界观树状图.xlsx
+++ b/瓶与井世界观树状图.xlsx
@@ -12,16 +12,18 @@
     <sheet name="1.1 赭锈带" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="1.2 陆海沙海" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="1.3 沙豚" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="2.1 污染主干" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="2.2 十三月" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="2.3 支线方案" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="3.1 生态酵母" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="3.2 燃料闭环" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="4. 历史脉络" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="5. 存在体谱系" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="6. 势力格局" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="7. 讽刺主题链" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="8. 叙事入口" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2.0 污染起因" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2.1 污染主干" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2.2 垦区源网" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2.3 十三月" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2.4 支线方案" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="3.1 生态酵母" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="3.2 燃料闭环" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="4. 历史脉络" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="5. 存在体谱系" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="6. 势力格局" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="7. 讽刺主题链" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="8. 叙事入口" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -482,7 +484,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》世界观树状图</t>
+          <t>《瓶与源》世界观树状图</t>
         </is>
       </c>
     </row>
@@ -494,7 +496,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-16-v7</t>
+          <t>2026-07-16-v8</t>
         </is>
       </c>
     </row>
@@ -518,7 +520,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>舞台 → 危机 → 技术 → 历史 → 存在体 → 势力 → 主题 → 入口</t>
+          <t>舞台 → 危机(起因+源网) → 技术 → 历史 → 存在体 → 势力 → 主题 → 入口</t>
         </is>
       </c>
     </row>
@@ -580,7 +582,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>《瓶与井》故事背景（垦历 C.Y. 42 · 十三月 Undecimber）</t>
+          <t>《瓶与源》故事背景（垦历 C.Y. 42 · 十三月 Undecimber）</t>
         </is>
       </c>
     </row>
@@ -594,7 +596,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【命题】掘井求生 → 造瓶产油</t>
+          <t xml:space="preserve">    ├─ 【命题】引源求生 → 造瓶产油</t>
         </is>
       </c>
     </row>
@@ -622,14 +624,14 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 边境殖民星 · 新西部社会 · 垦历 C.Y.</t>
+          <t xml:space="preserve">    │       ├─ 边境殖民星 · 卤缘渗出 · 冷凝塔网 · 垦区源网</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 陆海 / 沙海（重砂流态海 · 辐射尘富集）</t>
+          <t xml:space="preserve">    │       ├─ 陆海 / 沙海（重砂流态海 · 卤缘 · 辐射尘富集）</t>
         </is>
       </c>
     </row>
@@ -657,7 +659,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 化学层：深井毒卤（全年）</t>
+          <t xml:space="preserve">    │       ├─ 化学层：陆海卤缘渗出（全年）</t>
         </is>
       </c>
     </row>
@@ -671,208 +673,229 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 放射层：辐射尘（沙海扬尘 · Undecimber 叠加）</t>
+          <t xml:space="preserve">    │       ├─ 放射层：辐射尘（冷凝塔/源网 · Undecimber 叠加）</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 十三月 Undecimber ──→ 账外之月 · 全年最毒 · 觉醒临界</t>
+          <t xml:space="preserve">    │       ├─ 殖民诱因：卤缘渠网+冷凝并网 → 源网交叉污染</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    │       └─ 十三月 Undecimber ──→ 卤潮涨幅 · 全年最毒 · 觉醒临界</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【应答】生态酵母 Saccharomyces vitae</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 三重净化锈水 → 2–4% 生态酿（活命）</t>
+          <t xml:space="preserve">    ├─ 【应答】生态酵母 Saccharomyces vitae</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 二次发酵 → 40%+ 燃料乙醇（驱动世界）</t>
+          <t xml:space="preserve">    │       ├─ 三重净化锈水 → 2–4% 生态酿（活命）</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 谱系：W/R/F-Strain → 井兵 / 醇民 / 铁瓶 / 酿民</t>
+          <t xml:space="preserve">    │       ├─ 二次发酵 → 40%+ 燃料乙醇（驱动世界）</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    │       └─ 谱系：W/R/F-Strain → 滤兵 / 醇民 / 铁瓶 / 酿民</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【历史】C.Y. 5 锈水时代 → C.Y. 12 酵母 → C.Y. 23 铁瓶 → C.Y. 42 觉醒</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 【历史】C.Y. 5 锈水时代 → C.Y. 12 酵母 → C.Y. 23 铁瓶 → C.Y. 42 觉醒</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【存在体】井兵（平行）· 醇民 Gen-0（绝种）· 铁瓶 Gen-1 · 酿民 Gen-2</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 【存在体】滤兵（平行）· 醇民 Gen-0（绝种）· 铁瓶 Gen-1 · 酿民 Gen-2</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【势力】酿造帮 · 赏金猎人 · 戒酒教 · 流浪酒帮 · Saloon</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 【势力】酿造帮 · 赏金猎人 · 戒酒教 · 流浪酒帮 · Saloon</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    └─ 【当前】闭环运转 × 意识反抗 · 酒镇风暴眼 · 赤潮高峰</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>模块索引</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  01. 1.1 赭锈带</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  02. 1.2 陆海沙海</t>
+          <t xml:space="preserve">  01. 1.1 赭锈带</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  03. 1.3 沙豚</t>
+          <t xml:space="preserve">  02. 1.2 陆海沙海</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  04. 2.1 污染主干</t>
+          <t xml:space="preserve">  03. 1.3 沙豚</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  05. 2.2 十三月</t>
+          <t xml:space="preserve">  04. 2.0 污染起因</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  06. 2.3 支线方案</t>
+          <t xml:space="preserve">  05. 2.1 污染主干</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  07. 3.1 生态酵母</t>
+          <t xml:space="preserve">  06. 2.2 垦区源网</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  08. 3.2 燃料闭环</t>
+          <t xml:space="preserve">  07. 2.3 十三月</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  09. 4. 历史脉络</t>
+          <t xml:space="preserve">  08. 2.4 支线方案</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  10. 5. 存在体谱系</t>
+          <t xml:space="preserve">  09. 3.1 生态酵母</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  11. 6. 势力格局</t>
+          <t xml:space="preserve">  10. 3.2 燃料闭环</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  12. 7. 讽刺主题链</t>
+          <t xml:space="preserve">  11. 4. 历史脉络</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  13. 8. 叙事入口</t>
+          <t xml:space="preserve">  12. 5. 存在体谱系</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  13. 6. 势力格局</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  14. 7. 讽刺主题链</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  15. 8. 叙事入口</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="53">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A37:C37"/>
@@ -880,12 +903,14 @@
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A56:C56"/>
     <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A55:C55"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A57:C57"/>
     <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A42:C42"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A23:C23"/>
@@ -906,6 +931,7 @@
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A40:C40"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="A34:C34"/>
@@ -933,7 +959,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -944,14 +970,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 3.2 燃料闭环</t>
+          <t>《瓶与源》· 2.4 支线方案</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>燃料永续闭环（Fuel Perpetual Loop） ──→ C.Y. 23– · 铁瓶计划遗产</t>
+          <t>方案 A 陆海卤缘（Landsea Brine Rim） ──→ 推荐主干 · 盆地边缘天然卤渗出+卤缘渠网集中扩散</t>
         </is>
       </c>
     </row>
@@ -965,141 +991,41 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 输入层（Input Layer） ──→ C.Y. 23– · 锈水(锈卤+赤潮+辐射尘)、玉米浆、仙人掌糖浆</t>
+          <t xml:space="preserve">    └─ Undecimber 卤潮涨幅（Undecimber Brine Surge） ──→ 每年 · 陆海砂潮上涨，卤缘渗出率年度最高</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 地理层（Landsea Layer） ──→ 陆海重砂、辐射尘富集、野生铁瓶漂移带</t>
-        </is>
-      </c>
+      <c r="A6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 运输层（Transport Layer） ──→ C.Y. 25– · 饲料搬运者 Dust Walker</t>
+          <t>方案 B 流浪赤潮（Wandering Red Tide） ──→ 推荐叠加 · 嗜盐菌沿卤缘/源网季节性神经毒素</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 生产层（Production Layer） ──→ C.Y. 23– · 铁瓶 Synth-Bottle</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 一次发酵（Primary Fermentation） ──→ C.Y. 23– · 生态酿 2–4% 副产物</t>
+          <t xml:space="preserve">    └─ 赤潮高峰（Red Tide Peak） ──→ Undecimber · 全年水质最差月份</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │       └─ 二次发酵（Secondary Fermentation） ──→ C.Y. 23– · 燃料乙醇 40%+ 主产物</t>
-        </is>
-      </c>
+      <c r="A10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 输出层（Output Layer） ──→ C.Y. 23– · 机车、发电机、营地、Saloon</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 闭环裂缝（Loop Fracture） ──→ C.Y. 37+ · 二次发酵阈值，酿民觉醒</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与井》· 4. 历史脉络</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>锈水时代（Rustwater Era） ──→ C.Y. 5–12 · 深井卤锈化、Undecimber 赤潮、边境崩解</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>生态酵母问世（Eco-Yeast Discovery） ──→ C.Y. 12 Undecimber · 赭锈带首次现场验证</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>井源计划（Wellspring Program） ──→ C.Y. 12–17 · 首批植入净水士兵，C.Y. 14 战场验证</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 醇民 Gen-0 量产</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>泄露与抗争（Exposure &amp; Resistance） ──→ C.Y. 20–23 · Don't Bottle Humanity! 戒酒教萌芽</t>
+          <t>方案 C terraform 遗产（Terraform Legacy） ──→ 可选 · 早期大气改造站催化剂泄漏入源网</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1035,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23 Undecimber · 机械燃料解放人性，醇民销毁</t>
+          <t>方案 D 矿冶尾液（Smelting Tailings） ──→ 可选 · 炼矿尾液经支渠回流源网</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1045,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>机械时代（Mechanical Era） ──→ C.Y. 30–37 · 铁瓶量产，酿造帮商业化</t>
+          <t>方案 E 化武残留（Chemical War Residue） ──→ 可选 · 殖民内战化学剂污染支渠</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1055,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>酿民觉醒（Brewfolk Awakening） ──→ C.Y. 37–42 · 二次发酵阈值，瓶醒/井醒</t>
+          <t>方案 F 尘暴带电粒子（Dust Storm Ions） ──→ 可选 · 辐射尘机制的民间误传版本</t>
         </is>
       </c>
     </row>
@@ -1139,185 +1065,22 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>当前荒原（Present Wasteland） ──→ C.Y. 42 Undecimber · 闭环运转 × 意识反抗，赤潮高峰</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A15:C15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与井》· 5. 存在体谱系</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>井兵（Aqua-Soldiers） ──→ C.Y. 12– · 第一代植入者，W-Strain，平行谱系</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 归档者（The Archived） ──→ C.Y. 15– · 冷冻，记忆清洗</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 游荡老兵（The Dregs） ──→ C.Y. 15– · 荒漠传说，靠锈水存活</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 隐性血脉（Carrier Line） ──→ C.Y. 15– · 井醒来源</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉发酵容器，F-Strain，已灭绝</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识 android，F-Strain 机械舱</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 圈养牧场型（Ranch-Penned） ──→ C.Y. 23– · 酿造帮控制</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 野生游荡型（Wild Roaming） ──→ C.Y. 25– · 移动绿洲，赏金目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="7" t="inlineStr"/>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，数量大</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 井醒（Well-Awake） ──→ C.Y. 37+ · W-Strain 残留，数量少</t>
+          <t>推荐组合 A+B（Recommended A+B） ──→ 已并入主干 · 见「污染官方主干」模块</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 主流酿民派（Mainstream Brewfolk） ──→ C.Y. 37+ · 系统内求生</t>
-        </is>
-      </c>
+      <c r="A20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 流浪酒帮（Wander Brews） ──→ C.Y. 37+ · 脱离闭环</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 觉醒个体（Awakened Individuals） ──→ C.Y. 37+ · 独立思想者</t>
+          <t>生态酵母（统一应答）（Eco-Yeast Response） ──→ C.Y. 12– · 所有方案共同技术解：锈水→生态酿</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="20">
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A21:C21"/>
@@ -1325,7 +1088,6 @@
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A20:C20"/>
@@ -1344,7 +1106,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1360,14 +1122,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 6. 势力格局</t>
+          <t>《瓶与源》· 3.1 生态酵母</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>酿造帮（Stillwright Cartel） ──→ C.Y. 42 · 铁瓶遗产继承人，专利垄断，最大受益者</t>
+          <t>生态酵母（基础株）（Saccharomyces vitae） ──→ C.Y. 12– · 三重净化：化学毒+生物毒+辐射尘</t>
         </is>
       </c>
     </row>
@@ -1381,113 +1143,133 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 二次发酵专利（Secondary Fermentation IP） ──→ C.Y. 42 · 燃料乙醇 40%+ 垄断</t>
+          <t xml:space="preserve">    ├─ W-Strain（W-Strain (Military)） ──→ C.Y. 12–17 · 军用稳态型</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 商业化牧场（Commercial Ranches） ──→ C.Y. 42 · 圈养铁瓶，悬赏回收</t>
+          <t xml:space="preserve">    │   │</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 酿民回收令（Brewfolk Reclamation Order） ──→ C.Y. 42 · 觉醒酿民定义为废品</t>
+          <t xml:space="preserve">    │       └─ 源滤计划（Source-Filter Program） ──→ C.Y. 12–17 · 第一批植入者为锈水滤净士兵</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr"/>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │           │</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>赏金猎人（Bounty Hunters） ──→ C.Y. 42 · 回收野生铁瓶，猎捕叛逃酿民</t>
+          <t xml:space="preserve">    │           └─ 滤兵（Filter Soldiers） ──→ C.Y. 12–17 · 锈水→内源生态酿 2–4%</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    │               │</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 鏽釘（Rust Nail） ──→ C.Y. 42 · 职业猎人代表</t>
+          <t xml:space="preserve">    │               └─ 源醒（Source-Awake） ──→ C.Y. 37+ · W-Strain 残留 / 幸存滤兵</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 井兵单禁忌（Well-Soldier Taboo） ──→ C.Y. 42 · 圈内不接井兵委托</t>
+          <t xml:space="preserve">    ├─ R-Strain（R-Strain (Civilian)） ──→ C.Y. 12– · 民用救灾型</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="7" t="inlineStr"/>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │   │</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>戒酒教（Temperance Riders） ──→ C.Y. 42 · 早期禁酒主义 + 反改造宗教</t>
+          <t xml:space="preserve">    │       └─ 生态酿（Eco-Brew） ──→ C.Y. 12– · 2–4%，公开合法，社会认知「酵母=希望」</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    └─ F-Strain（F-Strain (Fuel)） ──→ C.Y. 15– · 燃料高产型</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 收割派（Harvest Faction） ──→ C.Y. 42 · 招募利用酿民，接口赎罪</t>
+          <t xml:space="preserve">        ├─ 活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 人体活体发酵容器</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 火焰纯净派（Flame Purity Faction） ──→ C.Y. 42 · 焚烧一切容器，铁瓶为伪善延续</t>
+          <t xml:space="preserve">        │   │</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="7" t="inlineStr"/>
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        │       └─ 醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉容器，已基本灭绝</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>流浪酒帮（Wander Brews） ──→ C.Y. 42 · 酿民反抗者，开源菌株，打破闭环</t>
+          <t xml:space="preserve">        └─ 铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23–30 · 菌株移植至机械载体</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="7" t="inlineStr"/>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                ├─ 铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识机械产力，圈养/野生</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>主流酿民派（Mainstream Brewfolk） ──→ C.Y. 42 · 系统内求生，仍辅助生产</t>
+          <t xml:space="preserve">                │   │</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="7" t="inlineStr"/>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            │       └─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，集体性觉醒</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>酒镇 / Saloon ──→ C.Y. 42 · 中立枢纽，情报，黑市，表面和平</t>
+          <t xml:space="preserve">                └─ 酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体，冲突中心</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1302,607 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 3.2 燃料闭环</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>燃料永续闭环（Fuel Perpetual Loop） ──→ C.Y. 23– · 铁瓶计划遗产</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 输入层（Input Layer） ──→ C.Y. 23– · 锈水(锈卤+赤潮+辐射尘)、玉米浆、仙人掌糖浆</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 地理层（Landsea Layer） ──→ 陆海重砂、辐射尘富集、野生铁瓶漂移带</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 运输层（Transport Layer） ──→ C.Y. 25– · 饲料搬运者 Dust Walker</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 生产层（Production Layer） ──→ C.Y. 23– · 铁瓶 Synth-Bottle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       ├─ 一次发酵（Primary Fermentation） ──→ C.Y. 23– · 生态酿 2–4% 副产物</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 二次发酵（Secondary Fermentation） ──→ C.Y. 23– · 燃料乙醇 40%+ 主产物</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 输出层（Output Layer） ──→ C.Y. 23– · 机车、发电机、营地、Saloon</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 闭环裂缝（Loop Fracture） ──→ C.Y. 37+ · 二次发酵阈值，酿民觉醒</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 4. 历史脉络</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>锈水时代（Rustwater Era） ──→ C.Y. 5–12 · 卤缘渠网并网、源网全域锈化、边境崩解</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>生态酵母问世（Eco-Yeast Discovery） ──→ C.Y. 12 Undecimber · 赭锈带首次现场验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>源滤计划（Source-Filter Program） ──→ C.Y. 12–17 · 首批植入滤兵，C.Y. 14 战场验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 醇民 Gen-0 量产</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>泄露与抗争（Exposure &amp; Resistance） ──→ C.Y. 20–23 · Don't Bottle Humanity! 戒酒教萌芽</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23 Undecimber · 机械燃料解放人性，醇民销毁</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>机械时代（Mechanical Era） ──→ C.Y. 30–37 · 铁瓶量产，酿造帮商业化</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>酿民觉醒（Brewfolk Awakening） ──→ C.Y. 37–42 · 二次发酵阈值，瓶醒/源醒</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>当前荒原（Present Wasteland） ──→ C.Y. 42 Undecimber · 闭环运转 × 意识反抗，赤潮高峰</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 5. 存在体谱系</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>滤兵（Filter Soldiers） ──→ C.Y. 12– · 第一代植入者，W-Strain，平行谱系</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 归档者（The Archived） ──→ C.Y. 15– · 冷冻，记忆清洗</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 游荡老兵（The Dregs） ──→ C.Y. 15– · 荒漠传说，靠锈水存活</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 隐性血脉（Carrier Line） ──→ C.Y. 15– · 源醒来源</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉发酵容器，F-Strain，已灭绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识 android，F-Strain 机械舱</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 圈养牧场型（Ranch-Penned） ──→ C.Y. 23– · 酿造帮控制</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 野生游荡型（Wild Roaming） ──→ C.Y. 25– · 移动绿洲，赏金目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，数量大</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 源醒（Source-Awake） ──→ C.Y. 37+ · W-Strain 残留，数量少</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 主流酿民派（Mainstream Brewfolk） ──→ C.Y. 37+ · 系统内求生</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 流浪酒帮（Wander Brews） ──→ C.Y. 37+ · 脱离闭环</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 觉醒个体（Awakened Individuals） ──→ C.Y. 37+ · 独立思想者</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 6. 势力格局</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>酿造帮（Stillwright Cartel） ──→ C.Y. 42 · 铁瓶遗产继承人，专利垄断，最大受益者</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 二次发酵专利（Secondary Fermentation IP） ──→ C.Y. 42 · 燃料乙醇 40%+ 垄断</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 商业化牧场（Commercial Ranches） ──→ C.Y. 42 · 圈养铁瓶，悬赏回收</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 酿民回收令（Brewfolk Reclamation Order） ──→ C.Y. 42 · 觉醒酿民定义为废品</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 否认源滤计划（Deny Source-Filter） ──→ C.Y. 42 · 档案抹除源滤计划历史</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>赏金猎人（Bounty Hunters） ──→ C.Y. 42 · 回收野生铁瓶，猎捕叛逃酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 鏽釘（Rust Nail） ──→ C.Y. 42 · 职业猎人代表</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 滤兵单禁忌（Filter-Soldier Taboo） ──→ C.Y. 42 · 圈内不接滤兵委托</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教（Temperance Riders） ──→ C.Y. 42 · 早期禁酒主义 + 反改造宗教</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 收割派（Harvest Faction） ──→ C.Y. 42 · 招募利用酿民，接口赎罪</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 火焰纯净派（Flame Purity Faction） ──→ C.Y. 42 · 焚烧一切容器，铁瓶为伪善延续</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>流浪酒帮（Wander Brews） ──→ C.Y. 42 · 酿民反抗者，开源菌株，打破闭环</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>主流酿民派（Mainstream Brewfolk） ──→ C.Y. 42 · 系统内求生，仍辅助生产</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>酒镇 / Saloon ──→ C.Y. 42 · 中立枢纽，情报，黑市，表面和平</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1536,7 +1918,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 7. 讽刺主题链</t>
+          <t>《瓶与源》· 7. 讽刺主题链</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1939,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 士兵净水（Soldiers Purify Water） ──→ C.Y. 12– · 最正当的起点</t>
+          <t xml:space="preserve">    └─ 士兵滤锈（Soldiers Filter Rustwater） ──→ C.Y. 12– · 最正当的起点</t>
         </is>
       </c>
     </row>
@@ -1668,7 +2050,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1684,14 +2066,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 8. 叙事入口</t>
+          <t>《瓶与源》· 8. 叙事入口</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>井兵末裔（Well-Soldier Scion） ──→ C.Y. 42 · W-Strain 残留，各方追逐</t>
+          <t>滤兵末裔（Filter-Soldier Scion） ──→ C.Y. 42 · W-Strain 残留，各方追逐</t>
         </is>
       </c>
     </row>
@@ -1701,7 +2083,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>刚觉醒酿民（Newly Awakened Brewfolk） ──→ C.Y. 42 · 意识到自己是净水者也是油箱</t>
+          <t>刚觉醒酿民（Newly Awakened Brewfolk） ──→ C.Y. 42 · 意识到自己是滤净者也是油箱</t>
         </is>
       </c>
     </row>
@@ -1711,7 +2093,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>鏽釘（Rust Nail） ──→ C.Y. 42 · 赏金猎人，禁忌井兵委托</t>
+          <t>鏽釘（Rust Nail） ──→ C.Y. 42 · 赏金猎人，禁忌滤兵委托</t>
         </is>
       </c>
     </row>
@@ -1758,7 +2140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C210"/>
+  <dimension ref="A1:C231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1769,7 +2151,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 全部树状图</t>
+          <t>《瓶与源》· 全部树状图</t>
         </is>
       </c>
     </row>
@@ -1811,7 +2193,7 @@
     <row r="8" outlineLevel="1" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 星球特征（Planet Traits） ──→ 双恒星、弱磁层、辐射尘、陆海沙海、稀薄大气</t>
+          <t xml:space="preserve">    ├─ 星球特征（Planet Traits） ──→ 双恒星、弱磁层、卤缘渗出、冷凝塔、陆海沙海</t>
         </is>
       </c>
     </row>
@@ -1888,35 +2270,35 @@
     <row r="20" outlineLevel="1" ht="16" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 辐射尘富集（Rad-Dust Enrichment） ──→ 辐射尘沉积于重砂层，翻涌时扬尘</t>
+          <t xml:space="preserve">    ├─ 卤缘 Brine Rim ──→ 盆地边缘天然卤渗出带，锈水化学层根源</t>
         </is>
       </c>
     </row>
     <row r="21" outlineLevel="1" ht="16" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 深井卤层出露（Brine Outcrop） ──→ 多数卤层出露点位于陆海盆地边缘</t>
+          <t xml:space="preserve">    ├─ 辐射尘富集（Rad-Dust Enrichment） ──→ 辐射尘沉积于重砂层，翻涌时扬尘</t>
         </is>
       </c>
     </row>
     <row r="22" outlineLevel="1" ht="16" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 殖民利用（Colonial Use） ──→ C.Y. 0– · 砂岸驿道、铁瓶牧场、非法酵母泥倾倒</t>
+          <t xml:space="preserve">    ├─ 殖民利用（Colonial Use） ──→ C.Y. 0– · 卤缘渠网、砂岸驿道、铁瓶牧场、酵母泥倾倒</t>
         </is>
       </c>
     </row>
     <row r="23" outlineLevel="1" ht="16" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 无井地带（Well-less Deep） ──→ 赏金猎人对陆海深处的称呼</t>
+          <t xml:space="preserve">    ├─ 无源地带（Source-less Deep） ──→ 赏金猎人对陆海深处的称呼</t>
         </is>
       </c>
     </row>
     <row r="24" outlineLevel="1" ht="16" customHeight="1">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 与锈水闭环（Rustwater Loop Link） ──→ 辐射尘+赤潮孢经砂层进入深井</t>
+          <t xml:space="preserve">    └─ 与锈水闭环（Rustwater Loop Link） ──→ 辐射尘+赤潮孢经砂层进入卤缘与源网</t>
         </is>
       </c>
     </row>
@@ -1958,7 +2340,7 @@
     <row r="31" outlineLevel="1" ht="16" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 集群迁徙（Herd Migration） ──→ Undecimber · 翻砂释放辐射尘与赤潮孢：沙豚起波井水变浊</t>
+          <t xml:space="preserve">    ├─ 集群迁徙（Herd Migration） ──→ Undecimber · 翻砂释放辐射尘与赤潮孢：沙豚起波源水变浊</t>
         </is>
       </c>
     </row>
@@ -1993,7 +2375,7 @@
     <row r="36" outlineLevel="1" ht="16" customHeight="1">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 第四镜像（Fourth Mirror） ──→ 对照井兵/铁瓶/酿民：自然进化不产酒</t>
+          <t xml:space="preserve">    ├─ 第四镜像（Fourth Mirror） ──→ 对照滤兵/铁瓶/酿民：自然进化不产酒</t>
         </is>
       </c>
     </row>
@@ -2007,14 +2389,14 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>▸ 2.1 污染主干</t>
+          <t>▸ 2.0 污染起因</t>
         </is>
       </c>
     </row>
     <row r="40" outlineLevel="1" ht="16" customHeight="1">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>官方主干 A+B+辐射尘（Canon A+B+Rad-Dust） ──→ 已定稿 · 三层污染叠加，生态酵母唯一规模化解</t>
+          <t>锈水成因链（Rustwater Causation） ──→ v8 定稿 · 先天本底+殖民并网放大+十三月时间层</t>
         </is>
       </c>
     </row>
@@ -2028,59 +2410,63 @@
     <row r="42" outlineLevel="1" ht="16" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 化学层 · 方案 A（Layer A Deep-Brine） ──→ 全年 · 深井卤层：高氯酸盐/砷/铜</t>
+          <t xml:space="preserve">    ├─ 先天层 · 星球本底（Primordial Layer） ──→ 卤缘天然有毒、嗜盐生态、弱磁辐射尘</t>
         </is>
       </c>
     </row>
     <row r="43" outlineLevel="1" ht="16" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 生物层 · 方案 B（Layer B Red Tide） ──→ Undecimber · 嗜盐菌神经毒素，水呈铁锈红浊</t>
+          <t xml:space="preserve">    ├─ 殖民层 · 人为放大（Colonial Amplification） ──→ C.Y. 2–12 · 卤缘渠网+冷凝塔并网→源网全域锈化</t>
         </is>
       </c>
     </row>
     <row r="44" outlineLevel="1" ht="16" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 放射层 · 辐射尘（Layer Rad-Dust） ──→ 尘暴/Undecimber · 轨道残骸+恒星风，沙海富集扬尘入水</t>
+          <t xml:space="preserve">    │       ├─ 卤缘渠网（Brine Rim Canals） ──→ C.Y. 2–8 · 沿陆海边缘截取天然卤渗出</t>
         </is>
       </c>
     </row>
     <row r="45" outlineLevel="1" ht="16" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ Undecimber 三重峰值（Triple Peak） ──→ Undecimber · 卤压+赤潮+辐射扬尘全年最毒</t>
+          <t xml:space="preserve">    │       ├─ 冷凝塔并网（Condenser Grid Merge） ──→ C.Y. 5–10 · 卤缘卤流与冷凝水并入同一源网</t>
         </is>
       </c>
     </row>
     <row r="46" outlineLevel="1" ht="16" customHeight="1">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 生态酵母三重净化（Eco-Yeast Triple Purify） ──→ C.Y. 12– · 钝化毒素+包裹核素→酵母泥需处置</t>
+          <t xml:space="preserve">    │       ├─ 源流未分级（No Source Segregation） ──→ C.Y. 5–12 · 误判稀释可管理毒性</t>
         </is>
       </c>
     </row>
     <row r="47" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A47" s="7" t="inlineStr"/>
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 支渠回流污染（Branch Canal Reflux） ──→ C.Y. 8–12 · 矿冶尾液、酵母泥渗漏回流</t>
+        </is>
+      </c>
     </row>
     <row r="48" outlineLevel="1" ht="16" customHeight="1">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>支线方案 C–F（Optional C–F） ──→ 局部 · 可作区域历史诱因，非主行星主干</t>
+          <t xml:space="preserve">    └─ 时间层 · 十三月（Undecimber Layer） ──→ 每年 · 卤潮涨幅+赤潮+辐射扬尘峰值</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>▸ 2.2 十三月</t>
+          <t>▸ 2.1 污染主干</t>
         </is>
       </c>
     </row>
     <row r="51" outlineLevel="1" ht="16" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>十三月 Undecimber ──→ 每年 37 垦日 · 垦历第 13 月，地球账本不承认</t>
+          <t>官方主干 A+B+辐射尘（Canon A+B+Rad-Dust） ──→ 已定稿 · 三层污染叠加，生态酵母唯一规模化解</t>
         </is>
       </c>
     </row>
@@ -2094,590 +2480,599 @@
     <row r="53" outlineLevel="1" ht="16" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 天文成因（Orbital Cause） ──→ 公转 397 垦日，余数并入第 13 月</t>
+          <t xml:space="preserve">    ├─ 化学层 · 方案 A（Layer A Brine Rim） ──→ 全年 · 陆海卤缘天然渗出+渠网集中扩散</t>
         </is>
       </c>
     </row>
     <row r="54" outlineLevel="1" ht="16" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 账外之月（Off-Ledger Month） ──→ 地球母公司不计 KPI 与编制</t>
+          <t xml:space="preserve">    ├─ 生物层 · 方案 B（Layer B Red Tide） ──→ Undecimber · 嗜盐菌沿卤缘/源网，神经毒素</t>
         </is>
       </c>
     </row>
     <row r="55" outlineLevel="1" ht="16" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 法外之月（Lawless Month） ──→ 悬赏翻倍、合同作废、黑市开市</t>
+          <t xml:space="preserve">    ├─ 放射层 · 辐射尘（Layer Rad-Dust） ──→ 尘暴/Undecimber · 冷凝塔、蓄源池、沙海扬尘</t>
         </is>
       </c>
     </row>
     <row r="56" outlineLevel="1" ht="16" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 水文峰值（Water Toxicity Peak） ──→ A+B+辐射尘 · 卤压+赤潮+沙海辐射扬尘</t>
+          <t xml:space="preserve">    ├─ Undecimber 三重峰值（Triple Peak） ──→ Undecimber · 卤潮涨幅+赤潮+辐射扬尘</t>
         </is>
       </c>
     </row>
     <row r="57" outlineLevel="1" ht="16" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ C.Y. 12 生态酵母验证（Yeast Field Test） ──→ C.Y. 12 · 首次现场验证生态酿</t>
+          <t xml:space="preserve">    └─ 生态酵母三重净化（Eco-Yeast Triple Purify） ──→ C.Y. 12– · 钝化毒素+包裹核素→酵母泥需处置</t>
         </is>
       </c>
     </row>
     <row r="58" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ C.Y. 12 井源计划植入（Wellspring Implant） ──→ C.Y. 12 · 首批净水士兵植入</t>
-        </is>
-      </c>
+      <c r="A58" s="7" t="inlineStr"/>
     </row>
     <row r="59" outlineLevel="1" ht="16" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ C.Y. 23 铁瓶招标截止（Synth-Bottle Tender） ──→ C.Y. 23 · 铁瓶计划招标在十三月截止</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ C.Y. 42 觉醒临界（Awakening Threshold） ──→ C.Y. 42 · 二次发酵阈值，当前叙事时点</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ Saloon 不打烊（Saloon Always Open） ──→ 整月营业，情报与黑市高峰</t>
+          <t>支线方案 C–F（Optional C–F） ──→ 局部 · 支渠污染或区域历史诱因</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>▸ 2.2 垦区源网</t>
         </is>
       </c>
     </row>
     <row r="62" outlineLevel="1" ht="16" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 酿造帮配额重置（Quota Reset） ──→ 年度生产配额于十三月 1 日重置</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="6" t="inlineStr">
-        <is>
-          <t>▸ 2.3 支线方案</t>
+          <t>垦区总水源网（Colonial Source Grid） ──→ C.Y. 2– · 非井模型 · 锈水在管网中流动分配</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 卤缘截取渠（Brine Rim Canals） ──→ C.Y. 2– · 沿陆海盆地边缘收集天然卤渗出</t>
         </is>
       </c>
     </row>
     <row r="65" outlineLevel="1" ht="16" customHeight="1">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>方案 A 深井毒卤（Deep-Brine Toxicity） ──→ 推荐主干 · 高氯酸盐/砷/铜卤层，深井采水全域污染</t>
+          <t xml:space="preserve">    ├─ 冷凝塔网（Condenser Towers） ──→ C.Y. 5– · 固陆砂岸高点集大气含水</t>
         </is>
       </c>
     </row>
     <row r="66" outlineLevel="1" ht="16" customHeight="1">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 蓄源池链（Reservoir Chain） ──→ C.Y. 5– · 卤缘水与冷凝水混合调蓄</t>
         </is>
       </c>
     </row>
     <row r="67" outlineLevel="1" ht="16" customHeight="1">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ Undecimber 卤压峰值（Undecimber Brine Peak） ──→ 每年 · 地下卤层渗透率年度最高</t>
+          <t xml:space="preserve">    ├─ 支渠与牧场接口（Branch Canals） ──→ C.Y. 8– · 牧场矿冶酵母泥处置回流支渠</t>
         </is>
       </c>
     </row>
     <row r="68" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A68" s="7" t="inlineStr"/>
-    </row>
-    <row r="69" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A69" s="7" t="inlineStr">
-        <is>
-          <t>方案 B 流浪赤潮（Wandering Red Tide） ──→ 推荐叠加 · 本土嗜盐菌季节性神经毒素</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 锈水 Rustwater ──→ 源网中一切流动储存分配的水体</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>▸ 2.3 十三月</t>
         </is>
       </c>
     </row>
     <row r="71" outlineLevel="1" ht="16" customHeight="1">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 赤潮高峰（Red Tide Peak） ──→ Undecimber · 全年水质最差月份</t>
+          <t>十三月 Undecimber ──→ 每年 37 垦日 · 垦历第 13 月，地球账本不承认</t>
         </is>
       </c>
     </row>
     <row r="72" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A72" s="7" t="inlineStr"/>
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="73" outlineLevel="1" ht="16" customHeight="1">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>方案 C terraform 遗产（Terraform Legacy） ──→ 可选 · 早期大气改造站催化剂泄漏</t>
+          <t xml:space="preserve">    ├─ 天文成因（Orbital Cause） ──→ 公转 397 垦日，余数并入第 13 月</t>
         </is>
       </c>
     </row>
     <row r="74" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A74" s="7" t="inlineStr"/>
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 账外之月（Off-Ledger Month） ──→ 地球母公司不计 KPI 与编制</t>
+        </is>
+      </c>
     </row>
     <row r="75" outlineLevel="1" ht="16" customHeight="1">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>方案 D 矿冶尾液（Smelting Tailings） ──→ 可选 · 机甲燃料炼矿尾液渗入含水层</t>
+          <t xml:space="preserve">    ├─ 法外之月（Lawless Month） ──→ 悬赏翻倍、合同作废、黑市开市</t>
         </is>
       </c>
     </row>
     <row r="76" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A76" s="7" t="inlineStr"/>
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 水文峰值（Water Toxicity Peak） ──→ A+B+辐射尘 · 卤潮涨幅+赤潮+沙海辐射扬尘</t>
+        </is>
+      </c>
     </row>
     <row r="77" outlineLevel="1" ht="16" customHeight="1">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>方案 E 化武残留（Chemical War Residue） ──→ 可选 · 殖民内战化学剂污染流域</t>
+          <t xml:space="preserve">    ├─ C.Y. 12 生态酵母验证（Yeast Field Test） ──→ C.Y. 12 · 首次现场验证生态酿</t>
         </is>
       </c>
     </row>
     <row r="78" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A78" s="7" t="inlineStr"/>
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ C.Y. 12 源滤计划植入（Source-Filter Implant） ──→ C.Y. 12 · 首批滤兵植入</t>
+        </is>
+      </c>
     </row>
     <row r="79" outlineLevel="1" ht="16" customHeight="1">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>方案 F 尘暴带电粒子（Dust Storm Ions） ──→ 可选 · 双恒星尘暴金属微粒随雨入水</t>
+          <t xml:space="preserve">    ├─ C.Y. 23 铁瓶招标截止（Synth-Bottle Tender） ──→ C.Y. 23 · 铁瓶计划招标在十三月截止</t>
         </is>
       </c>
     </row>
     <row r="80" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A80" s="7" t="inlineStr"/>
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ C.Y. 42 觉醒临界（Awakening Threshold） ──→ C.Y. 42 · 二次发酵阈值，当前叙事时点</t>
+        </is>
+      </c>
     </row>
     <row r="81" outlineLevel="1" ht="16" customHeight="1">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t>推荐组合 A+B（Recommended A+B） ──→ 已并入主干 · 见「污染官方主干」模块</t>
+          <t xml:space="preserve">    ├─ Saloon 不打烊（Saloon Always Open） ──→ 整月营业，情报与黑市高峰</t>
         </is>
       </c>
     </row>
     <row r="82" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A82" s="7" t="inlineStr"/>
-    </row>
-    <row r="83" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>生态酵母（统一应答）（Eco-Yeast Response） ──→ C.Y. 12– · 所有方案共同技术解：锈水→生态酿</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="6" t="inlineStr">
-        <is>
-          <t>▸ 3.1 生态酵母</t>
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 酿造帮配额重置（Quota Reset） ──→ 年度生产配额于十三月 1 日重置</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="inlineStr">
+        <is>
+          <t>▸ 2.4 支线方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>方案 A 陆海卤缘（Landsea Brine Rim） ──→ 推荐主干 · 盆地边缘天然卤渗出+卤缘渠网集中扩散</t>
         </is>
       </c>
     </row>
     <row r="86" outlineLevel="1" ht="16" customHeight="1">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>生态酵母（基础株）（Saccharomyces vitae） ──→ C.Y. 12– · 三重净化：化学毒+生物毒+辐射尘</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="87" outlineLevel="1" ht="16" customHeight="1">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    └─ Undecimber 卤潮涨幅（Undecimber Brine Surge） ──→ 每年 · 陆海砂潮上涨，卤缘渗出率年度最高</t>
         </is>
       </c>
     </row>
     <row r="88" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A88" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ W-Strain（W-Strain (Military)） ──→ C.Y. 12–17 · 军用稳态型</t>
-        </is>
-      </c>
+      <c r="A88" s="7" t="inlineStr"/>
     </row>
     <row r="89" outlineLevel="1" ht="16" customHeight="1">
       <c r="A89" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │   │</t>
+          <t>方案 B 流浪赤潮（Wandering Red Tide） ──→ 推荐叠加 · 嗜盐菌沿卤缘/源网季节性神经毒素</t>
         </is>
       </c>
     </row>
     <row r="90" outlineLevel="1" ht="16" customHeight="1">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 井源计划（Wellspring Program） ──→ C.Y. 12–17 · 第一批植入者为净水超级士兵</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="91" outlineLevel="1" ht="16" customHeight="1">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │           │</t>
+          <t xml:space="preserve">    └─ 赤潮高峰（Red Tide Peak） ──→ Undecimber · 全年水质最差月份</t>
         </is>
       </c>
     </row>
     <row r="92" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │           └─ 净水士兵（井兵）（Aqua-Soldiers） ──→ C.Y. 12–17 · 锈水→内源生态酿 2–4%</t>
-        </is>
-      </c>
+      <c r="A92" s="7" t="inlineStr"/>
     </row>
     <row r="93" outlineLevel="1" ht="16" customHeight="1">
       <c r="A93" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │               │</t>
+          <t>方案 C terraform 遗产（Terraform Legacy） ──→ 可选 · 早期大气改造站催化剂泄漏入源网</t>
         </is>
       </c>
     </row>
     <row r="94" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │               └─ 井醒（Well-Awake） ──→ C.Y. 37+ · W-Strain 残留 / 幸存井兵</t>
-        </is>
-      </c>
+      <c r="A94" s="7" t="inlineStr"/>
     </row>
     <row r="95" outlineLevel="1" ht="16" customHeight="1">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ R-Strain（R-Strain (Civilian)） ──→ C.Y. 12– · 民用救灾型</t>
+          <t>方案 D 矿冶尾液（Smelting Tailings） ──→ 可选 · 炼矿尾液经支渠回流源网</t>
         </is>
       </c>
     </row>
     <row r="96" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A96" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │   │</t>
-        </is>
-      </c>
+      <c r="A96" s="7" t="inlineStr"/>
     </row>
     <row r="97" outlineLevel="1" ht="16" customHeight="1">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 生态酿（Eco-Brew） ──→ C.Y. 12– · 2–4%，公开合法，社会认知「酵母=希望」</t>
+          <t>方案 E 化武残留（Chemical War Residue） ──→ 可选 · 殖民内战化学剂污染支渠</t>
         </is>
       </c>
     </row>
     <row r="98" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A98" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ F-Strain（F-Strain (Fuel)） ──→ C.Y. 15– · 燃料高产型</t>
-        </is>
-      </c>
+      <c r="A98" s="7" t="inlineStr"/>
     </row>
     <row r="99" outlineLevel="1" ht="16" customHeight="1">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ├─ 活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 人体活体发酵容器</t>
+          <t>方案 F 尘暴带电粒子（Dust Storm Ions） ──→ 可选 · 辐射尘机制的民间误传版本</t>
         </is>
       </c>
     </row>
     <row r="100" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A100" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        │   │</t>
-        </is>
-      </c>
+      <c r="A100" s="7" t="inlineStr"/>
     </row>
     <row r="101" outlineLevel="1" ht="16" customHeight="1">
       <c r="A101" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        │       └─ 醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉容器，已基本灭绝</t>
+          <t>推荐组合 A+B（Recommended A+B） ──→ 已并入主干 · 见「污染官方主干」模块</t>
         </is>
       </c>
     </row>
     <row r="102" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A102" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        └─ 铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23–30 · 菌株移植至机械载体</t>
-        </is>
-      </c>
+      <c r="A102" s="7" t="inlineStr"/>
     </row>
     <row r="103" outlineLevel="1" ht="16" customHeight="1">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                ├─ 铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识机械产力，圈养/野生</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A104" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                │   │</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A105" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            │       └─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，集体性觉醒</t>
+          <t>生态酵母（统一应答）（Eco-Yeast Response） ──→ C.Y. 12– · 所有方案共同技术解：锈水→生态酿</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>▸ 3.1 生态酵母</t>
         </is>
       </c>
     </row>
     <row r="106" outlineLevel="1" ht="16" customHeight="1">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                └─ 酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体，冲突中心</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>▸ 3.2 燃料闭环</t>
+          <t>生态酵母（基础株）（Saccharomyces vitae） ──→ C.Y. 12– · 三重净化：化学毒+生物毒+辐射尘</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ W-Strain（W-Strain (Military)） ──→ C.Y. 12–17 · 军用稳态型</t>
         </is>
       </c>
     </row>
     <row r="109" outlineLevel="1" ht="16" customHeight="1">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t>燃料永续闭环（Fuel Perpetual Loop） ──→ C.Y. 23– · 铁瓶计划遗产</t>
+          <t xml:space="preserve">    │   │</t>
         </is>
       </c>
     </row>
     <row r="110" outlineLevel="1" ht="16" customHeight="1">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    │       └─ 源滤计划（Source-Filter Program） ──→ C.Y. 12–17 · 第一批植入者为锈水滤净士兵</t>
         </is>
       </c>
     </row>
     <row r="111" outlineLevel="1" ht="16" customHeight="1">
       <c r="A111" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 输入层（Input Layer） ──→ C.Y. 23– · 锈水(锈卤+赤潮+辐射尘)、玉米浆、仙人掌糖浆</t>
+          <t xml:space="preserve">    │           │</t>
         </is>
       </c>
     </row>
     <row r="112" outlineLevel="1" ht="16" customHeight="1">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 地理层（Landsea Layer） ──→ 陆海重砂、辐射尘富集、野生铁瓶漂移带</t>
+          <t xml:space="preserve">    │           └─ 滤兵（Filter Soldiers） ──→ C.Y. 12–17 · 锈水→内源生态酿 2–4%</t>
         </is>
       </c>
     </row>
     <row r="113" outlineLevel="1" ht="16" customHeight="1">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 运输层（Transport Layer） ──→ C.Y. 25– · 饲料搬运者 Dust Walker</t>
+          <t xml:space="preserve">    │               │</t>
         </is>
       </c>
     </row>
     <row r="114" outlineLevel="1" ht="16" customHeight="1">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 生产层（Production Layer） ──→ C.Y. 23– · 铁瓶 Synth-Bottle</t>
+          <t xml:space="preserve">    │               └─ 源醒（Source-Awake） ──→ C.Y. 37+ · W-Strain 残留 / 幸存滤兵</t>
         </is>
       </c>
     </row>
     <row r="115" outlineLevel="1" ht="16" customHeight="1">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 一次发酵（Primary Fermentation） ──→ C.Y. 23– · 生态酿 2–4% 副产物</t>
+          <t xml:space="preserve">    ├─ R-Strain（R-Strain (Civilian)） ──→ C.Y. 12– · 民用救灾型</t>
         </is>
       </c>
     </row>
     <row r="116" outlineLevel="1" ht="16" customHeight="1">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 二次发酵（Secondary Fermentation） ──→ C.Y. 23– · 燃料乙醇 40%+ 主产物</t>
+          <t xml:space="preserve">    │   │</t>
         </is>
       </c>
     </row>
     <row r="117" outlineLevel="1" ht="16" customHeight="1">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 输出层（Output Layer） ──→ C.Y. 23– · 机车、发电机、营地、Saloon</t>
+          <t xml:space="preserve">    │       └─ 生态酿（Eco-Brew） ──→ C.Y. 12– · 2–4%，公开合法，社会认知「酵母=希望」</t>
         </is>
       </c>
     </row>
     <row r="118" outlineLevel="1" ht="16" customHeight="1">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 闭环裂缝（Loop Fracture） ──→ C.Y. 37+ · 二次发酵阈值，酿民觉醒</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="6" t="inlineStr">
-        <is>
-          <t>▸ 4. 历史脉络</t>
+          <t xml:space="preserve">    └─ F-Strain（F-Strain (Fuel)） ──→ C.Y. 15– · 燃料高产型</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ├─ 活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 人体活体发酵容器</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        │   │</t>
         </is>
       </c>
     </row>
     <row r="121" outlineLevel="1" ht="16" customHeight="1">
       <c r="A121" s="7" t="inlineStr">
         <is>
-          <t>锈水时代（Rustwater Era） ──→ C.Y. 5–12 · 深井卤锈化、Undecimber 赤潮、边境崩解</t>
+          <t xml:space="preserve">        │       └─ 醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉容器，已基本灭绝</t>
         </is>
       </c>
     </row>
     <row r="122" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A122" s="7" t="inlineStr"/>
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        └─ 铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23–30 · 菌株移植至机械载体</t>
+        </is>
+      </c>
     </row>
     <row r="123" outlineLevel="1" ht="16" customHeight="1">
       <c r="A123" s="7" t="inlineStr">
         <is>
-          <t>生态酵母问世（Eco-Yeast Discovery） ──→ C.Y. 12 Undecimber · 赭锈带首次现场验证</t>
+          <t xml:space="preserve">                ├─ 铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识机械产力，圈养/野生</t>
         </is>
       </c>
     </row>
     <row r="124" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A124" s="7" t="inlineStr"/>
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                │   │</t>
+        </is>
+      </c>
     </row>
     <row r="125" outlineLevel="1" ht="16" customHeight="1">
       <c r="A125" s="7" t="inlineStr">
         <is>
-          <t>井源计划（Wellspring Program） ──→ C.Y. 12–17 · 首批植入净水士兵，C.Y. 14 战场验证</t>
+          <t xml:space="preserve">            │       └─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，集体性觉醒</t>
         </is>
       </c>
     </row>
     <row r="126" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A126" s="7" t="inlineStr"/>
-    </row>
-    <row r="127" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A127" s="7" t="inlineStr">
-        <is>
-          <t>活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 醇民 Gen-0 量产</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A128" s="7" t="inlineStr"/>
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                └─ 酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体，冲突中心</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="6" t="inlineStr">
+        <is>
+          <t>▸ 3.2 燃料闭环</t>
+        </is>
+      </c>
     </row>
     <row r="129" outlineLevel="1" ht="16" customHeight="1">
       <c r="A129" s="7" t="inlineStr">
         <is>
-          <t>泄露与抗争（Exposure &amp; Resistance） ──→ C.Y. 20–23 · Don't Bottle Humanity! 戒酒教萌芽</t>
+          <t>燃料永续闭环（Fuel Perpetual Loop） ──→ C.Y. 23– · 铁瓶计划遗产</t>
         </is>
       </c>
     </row>
     <row r="130" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A130" s="7" t="inlineStr"/>
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="131" outlineLevel="1" ht="16" customHeight="1">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t>铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23 Undecimber · 机械燃料解放人性，醇民销毁</t>
+          <t xml:space="preserve">    ├─ 输入层（Input Layer） ──→ C.Y. 23– · 锈水(锈卤+赤潮+辐射尘)、玉米浆、仙人掌糖浆</t>
         </is>
       </c>
     </row>
     <row r="132" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A132" s="7" t="inlineStr"/>
+      <c r="A132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 地理层（Landsea Layer） ──→ 陆海重砂、辐射尘富集、野生铁瓶漂移带</t>
+        </is>
+      </c>
     </row>
     <row r="133" outlineLevel="1" ht="16" customHeight="1">
       <c r="A133" s="7" t="inlineStr">
         <is>
-          <t>机械时代（Mechanical Era） ──→ C.Y. 30–37 · 铁瓶量产，酿造帮商业化</t>
+          <t xml:space="preserve">    ├─ 运输层（Transport Layer） ──→ C.Y. 25– · 饲料搬运者 Dust Walker</t>
         </is>
       </c>
     </row>
     <row r="134" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A134" s="7" t="inlineStr"/>
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 生产层（Production Layer） ──→ C.Y. 23– · 铁瓶 Synth-Bottle</t>
+        </is>
+      </c>
     </row>
     <row r="135" outlineLevel="1" ht="16" customHeight="1">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>酿民觉醒（Brewfolk Awakening） ──→ C.Y. 37–42 · 二次发酵阈值，瓶醒/井醒</t>
+          <t xml:space="preserve">    │       ├─ 一次发酵（Primary Fermentation） ──→ C.Y. 23– · 生态酿 2–4% 副产物</t>
         </is>
       </c>
     </row>
     <row r="136" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A136" s="7" t="inlineStr"/>
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 二次发酵（Secondary Fermentation） ──→ C.Y. 23– · 燃料乙醇 40%+ 主产物</t>
+        </is>
+      </c>
     </row>
     <row r="137" outlineLevel="1" ht="16" customHeight="1">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>当前荒原（Present Wasteland） ──→ C.Y. 42 Undecimber · 闭环运转 × 意识反抗，赤潮高峰</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="6" t="inlineStr">
-        <is>
-          <t>▸ 5. 存在体谱系</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A140" s="7" t="inlineStr">
-        <is>
-          <t>井兵（Aqua-Soldiers） ──→ C.Y. 12– · 第一代植入者，W-Strain，平行谱系</t>
+          <t xml:space="preserve">    ├─ 输出层（Output Layer） ──→ C.Y. 23– · 机车、发电机、营地、Saloon</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 闭环裂缝（Loop Fracture） ──→ C.Y. 37+ · 二次发酵阈值，酿民觉醒</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="6" t="inlineStr">
+        <is>
+          <t>▸ 4. 历史脉络</t>
         </is>
       </c>
     </row>
     <row r="141" outlineLevel="1" ht="16" customHeight="1">
       <c r="A141" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>锈水时代（Rustwater Era） ──→ C.Y. 5–12 · 卤缘渠网并网、源网全域锈化、边境崩解</t>
         </is>
       </c>
     </row>
     <row r="142" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A142" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 归档者（The Archived） ──→ C.Y. 15– · 冷冻，记忆清洗</t>
-        </is>
-      </c>
+      <c r="A142" s="7" t="inlineStr"/>
     </row>
     <row r="143" outlineLevel="1" ht="16" customHeight="1">
       <c r="A143" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 游荡老兵（The Dregs） ──→ C.Y. 15– · 荒漠传说，靠锈水存活</t>
+          <t>生态酵母问世（Eco-Yeast Discovery） ──→ C.Y. 12 Undecimber · 赭锈带首次现场验证</t>
         </is>
       </c>
     </row>
     <row r="144" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A144" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 隐性血脉（Carrier Line） ──→ C.Y. 15– · 井醒来源</t>
-        </is>
-      </c>
+      <c r="A144" s="7" t="inlineStr"/>
     </row>
     <row r="145" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A145" s="7" t="inlineStr"/>
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>源滤计划（Source-Filter Program） ──→ C.Y. 12–17 · 首批植入滤兵，C.Y. 14 战场验证</t>
+        </is>
+      </c>
     </row>
     <row r="146" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A146" s="7" t="inlineStr">
-        <is>
-          <t>醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉发酵容器，F-Strain，已灭绝</t>
-        </is>
-      </c>
+      <c r="A146" s="7" t="inlineStr"/>
     </row>
     <row r="147" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A147" s="7" t="inlineStr"/>
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t>活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 醇民 Gen-0 量产</t>
+        </is>
+      </c>
     </row>
     <row r="148" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A148" s="7" t="inlineStr">
-        <is>
-          <t>铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识 android，F-Strain 机械舱</t>
-        </is>
-      </c>
+      <c r="A148" s="7" t="inlineStr"/>
     </row>
     <row r="149" outlineLevel="1" ht="16" customHeight="1">
       <c r="A149" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>泄露与抗争（Exposure &amp; Resistance） ──→ C.Y. 20–23 · Don't Bottle Humanity! 戒酒教萌芽</t>
         </is>
       </c>
     </row>
     <row r="150" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A150" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 圈养牧场型（Ranch-Penned） ──→ C.Y. 23– · 酿造帮控制</t>
-        </is>
-      </c>
+      <c r="A150" s="7" t="inlineStr"/>
     </row>
     <row r="151" outlineLevel="1" ht="16" customHeight="1">
       <c r="A151" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 野生游荡型（Wild Roaming） ──→ C.Y. 25– · 移动绿洲，赏金目标</t>
+          <t>铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23 Undecimber · 机械燃料解放人性，醇民销毁</t>
         </is>
       </c>
     </row>
@@ -2687,91 +3082,79 @@
     <row r="153" outlineLevel="1" ht="16" customHeight="1">
       <c r="A153" s="7" t="inlineStr">
         <is>
-          <t>酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体</t>
+          <t>机械时代（Mechanical Era） ──→ C.Y. 30–37 · 铁瓶量产，酿造帮商业化</t>
         </is>
       </c>
     </row>
     <row r="154" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A154" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
+      <c r="A154" s="7" t="inlineStr"/>
     </row>
     <row r="155" outlineLevel="1" ht="16" customHeight="1">
       <c r="A155" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，数量大</t>
+          <t>酿民觉醒（Brewfolk Awakening） ──→ C.Y. 37–42 · 二次发酵阈值，瓶醒/源醒</t>
         </is>
       </c>
     </row>
     <row r="156" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A156" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 井醒（Well-Awake） ──→ C.Y. 37+ · W-Strain 残留，数量少</t>
-        </is>
-      </c>
+      <c r="A156" s="7" t="inlineStr"/>
     </row>
     <row r="157" outlineLevel="1" ht="16" customHeight="1">
       <c r="A157" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 主流酿民派（Mainstream Brewfolk） ──→ C.Y. 37+ · 系统内求生</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A158" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 流浪酒帮（Wander Brews） ──→ C.Y. 37+ · 脱离闭环</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A159" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 觉醒个体（Awakened Individuals） ──→ C.Y. 37+ · 独立思想者</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="6" t="inlineStr">
-        <is>
-          <t>▸ 6. 势力格局</t>
+          <t>当前荒原（Present Wasteland） ──→ C.Y. 42 Undecimber · 闭环运转 × 意识反抗，赤潮高峰</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>▸ 5. 存在体谱系</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A160" s="7" t="inlineStr">
+        <is>
+          <t>滤兵（Filter Soldiers） ──→ C.Y. 12– · 第一代植入者，W-Strain，平行谱系</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A161" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="162" outlineLevel="1" ht="16" customHeight="1">
       <c r="A162" s="7" t="inlineStr">
         <is>
-          <t>酿造帮（Stillwright Cartel） ──→ C.Y. 42 · 铁瓶遗产继承人，专利垄断，最大受益者</t>
+          <t xml:space="preserve">    ├─ 归档者（The Archived） ──→ C.Y. 15– · 冷冻，记忆清洗</t>
         </is>
       </c>
     </row>
     <row r="163" outlineLevel="1" ht="16" customHeight="1">
       <c r="A163" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 游荡老兵（The Dregs） ──→ C.Y. 15– · 荒漠传说，靠锈水存活</t>
         </is>
       </c>
     </row>
     <row r="164" outlineLevel="1" ht="16" customHeight="1">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 二次发酵专利（Secondary Fermentation IP） ──→ C.Y. 42 · 燃料乙醇 40%+ 垄断</t>
+          <t xml:space="preserve">    └─ 隐性血脉（Carrier Line） ──→ C.Y. 15– · 源醒来源</t>
         </is>
       </c>
     </row>
     <row r="165" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A165" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 商业化牧场（Commercial Ranches） ──→ C.Y. 42 · 圈养铁瓶，悬赏回收</t>
-        </is>
-      </c>
+      <c r="A165" s="7" t="inlineStr"/>
     </row>
     <row r="166" outlineLevel="1" ht="16" customHeight="1">
       <c r="A166" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 酿民回收令（Brewfolk Reclamation Order） ──→ C.Y. 42 · 觉醒酿民定义为废品</t>
+          <t>醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉发酵容器，F-Strain，已灭绝</t>
         </is>
       </c>
     </row>
@@ -2781,7 +3164,7 @@
     <row r="168" outlineLevel="1" ht="16" customHeight="1">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t>赏金猎人（Bounty Hunters） ──→ C.Y. 42 · 回收野生铁瓶，猎捕叛逃酿民</t>
+          <t>铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识 android，F-Strain 机械舱</t>
         </is>
       </c>
     </row>
@@ -2795,14 +3178,14 @@
     <row r="170" outlineLevel="1" ht="16" customHeight="1">
       <c r="A170" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 鏽釘（Rust Nail） ──→ C.Y. 42 · 职业猎人代表</t>
+          <t xml:space="preserve">    ├─ 圈养牧场型（Ranch-Penned） ──→ C.Y. 23– · 酿造帮控制</t>
         </is>
       </c>
     </row>
     <row r="171" outlineLevel="1" ht="16" customHeight="1">
       <c r="A171" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 井兵单禁忌（Well-Soldier Taboo） ──→ C.Y. 42 · 圈内不接井兵委托</t>
+          <t xml:space="preserve">    └─ 野生游荡型（Wild Roaming） ──→ C.Y. 25– · 移动绿洲，赏金目标</t>
         </is>
       </c>
     </row>
@@ -2812,7 +3195,7 @@
     <row r="173" outlineLevel="1" ht="16" customHeight="1">
       <c r="A173" s="7" t="inlineStr">
         <is>
-          <t>戒酒教（Temperance Riders） ──→ C.Y. 42 · 早期禁酒主义 + 反改造宗教</t>
+          <t>酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体</t>
         </is>
       </c>
     </row>
@@ -2826,215 +3209,347 @@
     <row r="175" outlineLevel="1" ht="16" customHeight="1">
       <c r="A175" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 收割派（Harvest Faction） ──→ C.Y. 42 · 招募利用酿民，接口赎罪</t>
+          <t xml:space="preserve">    ├─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，数量大</t>
         </is>
       </c>
     </row>
     <row r="176" outlineLevel="1" ht="16" customHeight="1">
       <c r="A176" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 火焰纯净派（Flame Purity Faction） ──→ C.Y. 42 · 焚烧一切容器，铁瓶为伪善延续</t>
+          <t xml:space="preserve">    ├─ 源醒（Source-Awake） ──→ C.Y. 37+ · W-Strain 残留，数量少</t>
         </is>
       </c>
     </row>
     <row r="177" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A177" s="7" t="inlineStr"/>
+      <c r="A177" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 主流酿民派（Mainstream Brewfolk） ──→ C.Y. 37+ · 系统内求生</t>
+        </is>
+      </c>
     </row>
     <row r="178" outlineLevel="1" ht="16" customHeight="1">
       <c r="A178" s="7" t="inlineStr">
         <is>
-          <t>流浪酒帮（Wander Brews） ──→ C.Y. 42 · 酿民反抗者，开源菌株，打破闭环</t>
+          <t xml:space="preserve">    ├─ 流浪酒帮（Wander Brews） ──→ C.Y. 37+ · 脱离闭环</t>
         </is>
       </c>
     </row>
     <row r="179" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A179" s="7" t="inlineStr"/>
-    </row>
-    <row r="180" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A180" s="7" t="inlineStr">
-        <is>
-          <t>主流酿民派（Mainstream Brewfolk） ──→ C.Y. 42 · 系统内求生，仍辅助生产</t>
-        </is>
-      </c>
-    </row>
-    <row r="181" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A181" s="7" t="inlineStr"/>
+      <c r="A179" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 觉醒个体（Awakened Individuals） ──→ C.Y. 37+ · 独立思想者</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="6" t="inlineStr">
+        <is>
+          <t>▸ 6. 势力格局</t>
+        </is>
+      </c>
     </row>
     <row r="182" outlineLevel="1" ht="16" customHeight="1">
       <c r="A182" s="7" t="inlineStr">
         <is>
-          <t>酒镇 / Saloon ──→ C.Y. 42 · 中立枢纽，情报，黑市，表面和平</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="6" t="inlineStr">
-        <is>
-          <t>▸ 7. 讽刺主题链</t>
+          <t>酿造帮（Stillwright Cartel） ──→ C.Y. 42 · 铁瓶遗产继承人，专利垄断，最大受益者</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A184" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 二次发酵专利（Secondary Fermentation IP） ──→ C.Y. 42 · 燃料乙醇 40%+ 垄断</t>
         </is>
       </c>
     </row>
     <row r="185" outlineLevel="1" ht="16" customHeight="1">
       <c r="A185" s="7" t="inlineStr">
         <is>
-          <t>旧时代生存执念（Survival Obsession） ──→ 无论如何都要活下去</t>
+          <t xml:space="preserve">    ├─ 商业化牧场（Commercial Ranches） ──→ C.Y. 42 · 圈养铁瓶，悬赏回收</t>
         </is>
       </c>
     </row>
     <row r="186" outlineLevel="1" ht="16" customHeight="1">
       <c r="A186" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 酿民回收令（Brewfolk Reclamation Order） ──→ C.Y. 42 · 觉醒酿民定义为废品</t>
         </is>
       </c>
     </row>
     <row r="187" outlineLevel="1" ht="16" customHeight="1">
       <c r="A187" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 士兵净水（Soldiers Purify Water） ──→ C.Y. 12– · 最正当的起点</t>
+          <t xml:space="preserve">    └─ 否认源滤计划（Deny Source-Filter） ──→ C.Y. 42 · 档案抹除源滤计划历史</t>
         </is>
       </c>
     </row>
     <row r="188" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A188" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        │</t>
-        </is>
-      </c>
+      <c r="A188" s="7" t="inlineStr"/>
     </row>
     <row r="189" outlineLevel="1" ht="16" customHeight="1">
       <c r="A189" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        └─ 人体验证（Human Vessel Proven） ──→ C.Y. 14– · 技术门槛跨越</t>
+          <t>赏金猎人（Bounty Hunters） ──→ C.Y. 42 · 回收野生铁瓶，猎捕叛逃酿民</t>
         </is>
       </c>
     </row>
     <row r="190" outlineLevel="1" ht="16" customHeight="1">
       <c r="A190" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">            │</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="191" outlineLevel="1" ht="16" customHeight="1">
       <c r="A191" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                └─ 贫民燃料化（Poor as Fuel） ──→ C.Y. 15– · 对象降级，话术不变</t>
+          <t xml:space="preserve">    ├─ 鏽釘（Rust Nail） ──→ C.Y. 42 · 职业猎人代表</t>
         </is>
       </c>
     </row>
     <row r="192" outlineLevel="1" ht="16" customHeight="1">
       <c r="A192" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                    │</t>
+          <t xml:space="preserve">    └─ 滤兵单禁忌（Filter-Soldier Taboo） ──→ C.Y. 42 · 圈内不接滤兵委托</t>
         </is>
       </c>
     </row>
     <row r="193" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A193" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                    └─ 人道抗争（Humanitarian Protest） ──→ C.Y. 20– · 别把人变成瓶子</t>
-        </is>
-      </c>
+      <c r="A193" s="7" t="inlineStr"/>
     </row>
     <row r="194" outlineLevel="1" ht="16" customHeight="1">
       <c r="A194" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                        │</t>
+          <t>戒酒教（Temperance Riders） ──→ C.Y. 42 · 早期禁酒主义 + 反改造宗教</t>
         </is>
       </c>
     </row>
     <row r="195" outlineLevel="1" ht="16" customHeight="1">
       <c r="A195" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                        └─ 铁瓶妥协（Synth-Bottle Compromise） ──→ C.Y. 23– · 机械燃料，解放人性</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="196" outlineLevel="1" ht="16" customHeight="1">
       <c r="A196" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                            │</t>
+          <t xml:space="preserve">    ├─ 收割派（Harvest Faction） ──→ C.Y. 42 · 招募利用酿民，接口赎罪</t>
         </is>
       </c>
     </row>
     <row r="197" outlineLevel="1" ht="16" customHeight="1">
       <c r="A197" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                            └─ 机械量产（Mass Production） ──→ C.Y. 30– · 人性换效率</t>
+          <t xml:space="preserve">    └─ 火焰纯净派（Flame Purity Faction） ──→ C.Y. 42 · 焚烧一切容器，铁瓶为伪善延续</t>
         </is>
       </c>
     </row>
     <row r="198" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A198" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                                │</t>
-        </is>
-      </c>
+      <c r="A198" s="7" t="inlineStr"/>
     </row>
     <row r="199" outlineLevel="1" ht="16" customHeight="1">
       <c r="A199" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">                                └─ 酿民觉醒（Brewfolk Awakening） ──→ C.Y. 37+ · 容器发问，闭环裂缝</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="6" t="inlineStr">
-        <is>
-          <t>▸ 8. 叙事入口</t>
+          <t>流浪酒帮（Wander Brews） ──→ C.Y. 42 · 酿民反抗者，开源菌株，打破闭环</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A200" s="7" t="inlineStr"/>
+    </row>
+    <row r="201" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A201" s="7" t="inlineStr">
+        <is>
+          <t>主流酿民派（Mainstream Brewfolk） ──→ C.Y. 42 · 系统内求生，仍辅助生产</t>
         </is>
       </c>
     </row>
     <row r="202" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A202" s="7" t="inlineStr">
-        <is>
-          <t>井兵末裔（Well-Soldier Scion） ──→ C.Y. 42 · W-Strain 残留，各方追逐</t>
-        </is>
-      </c>
+      <c r="A202" s="7" t="inlineStr"/>
     </row>
     <row r="203" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A203" s="7" t="inlineStr"/>
-    </row>
-    <row r="204" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A204" s="7" t="inlineStr">
-        <is>
-          <t>刚觉醒酿民（Newly Awakened Brewfolk） ──→ C.Y. 42 · 意识到自己是净水者也是油箱</t>
-        </is>
-      </c>
-    </row>
-    <row r="205" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A205" s="7" t="inlineStr"/>
+      <c r="A203" s="7" t="inlineStr">
+        <is>
+          <t>酒镇 / Saloon ──→ C.Y. 42 · 中立枢纽，情报，黑市，表面和平</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="6" t="inlineStr">
+        <is>
+          <t>▸ 7. 讽刺主题链</t>
+        </is>
+      </c>
     </row>
     <row r="206" outlineLevel="1" ht="16" customHeight="1">
       <c r="A206" s="7" t="inlineStr">
         <is>
-          <t>鏽釘（Rust Nail） ──→ C.Y. 42 · 赏金猎人，禁忌井兵委托</t>
+          <t>旧时代生存执念（Survival Obsession） ──→ 无论如何都要活下去</t>
         </is>
       </c>
     </row>
     <row r="207" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A207" s="7" t="inlineStr"/>
+      <c r="A207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="208" outlineLevel="1" ht="16" customHeight="1">
       <c r="A208" s="7" t="inlineStr">
         <is>
-          <t>Saloon 酒保（Saloon Bartender） ──→ C.Y. 42 · 半觉醒老旧铁瓶</t>
+          <t xml:space="preserve">    └─ 士兵滤锈（Soldiers Filter Rustwater） ──→ C.Y. 12– · 最正当的起点</t>
         </is>
       </c>
     </row>
     <row r="209" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A209" s="7" t="inlineStr"/>
+      <c r="A209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        │</t>
+        </is>
+      </c>
     </row>
     <row r="210" outlineLevel="1" ht="16" customHeight="1">
       <c r="A210" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">        └─ 人体验证（Human Vessel Proven） ──→ C.Y. 14– · 技术门槛跨越</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            │</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                └─ 贫民燃料化（Poor as Fuel） ──→ C.Y. 15– · 对象降级，话术不变</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    └─ 人道抗争（Humanitarian Protest） ──→ C.Y. 20– · 别把人变成瓶子</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A215" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                        │</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                        └─ 铁瓶妥协（Synth-Bottle Compromise） ──→ C.Y. 23– · 机械燃料，解放人性</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                            │</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                            └─ 机械量产（Mass Production） ──→ C.Y. 30– · 人性换效率</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                │</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                └─ 酿民觉醒（Brewfolk Awakening） ──→ C.Y. 37+ · 容器发问，闭环裂缝</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="6" t="inlineStr">
+        <is>
+          <t>▸ 8. 叙事入口</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A223" s="7" t="inlineStr">
+        <is>
+          <t>滤兵末裔（Filter-Soldier Scion） ──→ C.Y. 42 · W-Strain 残留，各方追逐</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A224" s="7" t="inlineStr"/>
+    </row>
+    <row r="225" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A225" s="7" t="inlineStr">
+        <is>
+          <t>刚觉醒酿民（Newly Awakened Brewfolk） ──→ C.Y. 42 · 意识到自己是滤净者也是油箱</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A226" s="7" t="inlineStr"/>
+    </row>
+    <row r="227" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A227" s="7" t="inlineStr">
+        <is>
+          <t>鏽釘（Rust Nail） ──→ C.Y. 42 · 赏金猎人，禁忌滤兵委托</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A228" s="7" t="inlineStr"/>
+    </row>
+    <row r="229" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A229" s="7" t="inlineStr">
+        <is>
+          <t>Saloon 酒保（Saloon Bartender） ──→ C.Y. 42 · 半觉醒老旧铁瓶</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A230" s="7" t="inlineStr"/>
+    </row>
+    <row r="231" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A231" s="7" t="inlineStr">
+        <is>
           <t>酿造帮档案员（Cartel Archivist） ──→ C.Y. 42 · 发现抗议领袖在铁瓶合同上</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="197">
+  <mergeCells count="216">
     <mergeCell ref="A128:C128"/>
     <mergeCell ref="A193:C193"/>
     <mergeCell ref="A80:C80"/>
@@ -3063,22 +3578,27 @@
     <mergeCell ref="A171:C171"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="A165:C165"/>
+    <mergeCell ref="A63:C63"/>
     <mergeCell ref="A155:C155"/>
     <mergeCell ref="A93:C93"/>
+    <mergeCell ref="A220:C220"/>
     <mergeCell ref="A173:C173"/>
+    <mergeCell ref="A229:C229"/>
     <mergeCell ref="A130:C130"/>
     <mergeCell ref="A77:C77"/>
     <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A83:C83"/>
     <mergeCell ref="A148:C148"/>
     <mergeCell ref="A157:C157"/>
+    <mergeCell ref="A222:C222"/>
+    <mergeCell ref="A138:C138"/>
     <mergeCell ref="A132:C132"/>
     <mergeCell ref="A110:C110"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A119:C119"/>
     <mergeCell ref="A196:C196"/>
     <mergeCell ref="A174:C174"/>
     <mergeCell ref="A205:C205"/>
+    <mergeCell ref="A183:C183"/>
     <mergeCell ref="A66:C66"/>
     <mergeCell ref="A118:C118"/>
     <mergeCell ref="A75:C75"/>
@@ -3088,15 +3608,18 @@
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A95:C95"/>
-    <mergeCell ref="A104:C104"/>
+    <mergeCell ref="A160:C160"/>
     <mergeCell ref="A175:C175"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A159:C159"/>
     <mergeCell ref="A97:C97"/>
+    <mergeCell ref="A219:C219"/>
+    <mergeCell ref="A224:C224"/>
     <mergeCell ref="A106:C106"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A200:C200"/>
     <mergeCell ref="A81:C81"/>
     <mergeCell ref="A96:C96"/>
     <mergeCell ref="A209:C209"/>
@@ -3110,6 +3633,7 @@
     <mergeCell ref="A202:C202"/>
     <mergeCell ref="A58:C58"/>
     <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A211:C211"/>
     <mergeCell ref="A67:C67"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A186:C186"/>
@@ -3118,28 +3642,32 @@
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A201:C201"/>
     <mergeCell ref="A82:C82"/>
-    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="A226:C226"/>
     <mergeCell ref="A123:C123"/>
     <mergeCell ref="A197:C197"/>
+    <mergeCell ref="A228:C228"/>
     <mergeCell ref="A146:C146"/>
     <mergeCell ref="A124:C124"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A172:C172"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A187:C187"/>
+    <mergeCell ref="A212:C212"/>
     <mergeCell ref="A99:C99"/>
     <mergeCell ref="A108:C108"/>
+    <mergeCell ref="A84:C84"/>
     <mergeCell ref="A149:C149"/>
+    <mergeCell ref="A214:C214"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A163:C163"/>
-    <mergeCell ref="A158:C158"/>
+    <mergeCell ref="A189:C189"/>
     <mergeCell ref="A101:C101"/>
-    <mergeCell ref="A189:C189"/>
+    <mergeCell ref="A223:C223"/>
     <mergeCell ref="A50:C50"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A86:C86"/>
-    <mergeCell ref="A204:C204"/>
     <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A213:C213"/>
     <mergeCell ref="A151:C151"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A188:C188"/>
@@ -3152,6 +3680,7 @@
     <mergeCell ref="A62:C62"/>
     <mergeCell ref="A144:C144"/>
     <mergeCell ref="A122:C122"/>
+    <mergeCell ref="A215:C215"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A125:C125"/>
     <mergeCell ref="A190:C190"/>
@@ -3161,7 +3690,6 @@
     <mergeCell ref="A112:C112"/>
     <mergeCell ref="A199:C199"/>
     <mergeCell ref="A152:C152"/>
-    <mergeCell ref="A127:C127"/>
     <mergeCell ref="A167:C167"/>
     <mergeCell ref="A176:C176"/>
     <mergeCell ref="A30:C30"/>
@@ -3172,6 +3700,8 @@
     <mergeCell ref="A98:C98"/>
     <mergeCell ref="A191:C191"/>
     <mergeCell ref="A169:C169"/>
+    <mergeCell ref="A225:C225"/>
+    <mergeCell ref="A107:C107"/>
     <mergeCell ref="A178:C178"/>
     <mergeCell ref="A79:C79"/>
     <mergeCell ref="A61:C61"/>
@@ -3179,17 +3709,18 @@
     <mergeCell ref="A70:C70"/>
     <mergeCell ref="A153:C153"/>
     <mergeCell ref="A162:C162"/>
+    <mergeCell ref="A227:C227"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="A137:C137"/>
     <mergeCell ref="A177:C177"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A90:C90"/>
+    <mergeCell ref="A217:C217"/>
     <mergeCell ref="A164:C164"/>
     <mergeCell ref="A74:C74"/>
     <mergeCell ref="A56:C56"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A145:C145"/>
-    <mergeCell ref="A139:C139"/>
     <mergeCell ref="A154:C154"/>
     <mergeCell ref="A129:C129"/>
     <mergeCell ref="A195:C195"/>
@@ -3206,13 +3737,14 @@
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="A109:C109"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A180:C180"/>
+    <mergeCell ref="A231:C231"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A115:C115"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A68:C68"/>
     <mergeCell ref="A102:C102"/>
     <mergeCell ref="A117:C117"/>
+    <mergeCell ref="A230:C230"/>
     <mergeCell ref="A111:C111"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A143:C143"/>
@@ -3228,10 +3760,12 @@
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A94:C94"/>
     <mergeCell ref="A103:C103"/>
+    <mergeCell ref="A216:C216"/>
     <mergeCell ref="A168:C168"/>
     <mergeCell ref="A78:C78"/>
     <mergeCell ref="A87:C87"/>
     <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A218:C218"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3253,7 +3787,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 1.1 赭锈带</t>
+          <t>《瓶与源》· 1.1 赭锈带</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3815,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 星球特征（Planet Traits） ──→ 双恒星、弱磁层、辐射尘、陆海沙海、稀薄大气</t>
+          <t xml:space="preserve">    ├─ 星球特征（Planet Traits） ──→ 双恒星、弱磁层、卤缘渗出、冷凝塔、陆海沙海</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3887,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 1.2 陆海沙海</t>
+          <t>《瓶与源》· 1.2 陆海沙海</t>
         </is>
       </c>
     </row>
@@ -3388,35 +3922,35 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 辐射尘富集（Rad-Dust Enrichment） ──→ 辐射尘沉积于重砂层，翻涌时扬尘</t>
+          <t xml:space="preserve">    ├─ 卤缘 Brine Rim ──→ 盆地边缘天然卤渗出带，锈水化学层根源</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 深井卤层出露（Brine Outcrop） ──→ 多数卤层出露点位于陆海盆地边缘</t>
+          <t xml:space="preserve">    ├─ 辐射尘富集（Rad-Dust Enrichment） ──→ 辐射尘沉积于重砂层，翻涌时扬尘</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 殖民利用（Colonial Use） ──→ C.Y. 0– · 砂岸驿道、铁瓶牧场、非法酵母泥倾倒</t>
+          <t xml:space="preserve">    ├─ 殖民利用（Colonial Use） ──→ C.Y. 0– · 卤缘渠网、砂岸驿道、铁瓶牧场、酵母泥倾倒</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 无井地带（Well-less Deep） ──→ 赏金猎人对陆海深处的称呼</t>
+          <t xml:space="preserve">    ├─ 无源地带（Source-less Deep） ──→ 赏金猎人对陆海深处的称呼</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 与锈水闭环（Rustwater Loop Link） ──→ 辐射尘+赤潮孢经砂层进入深井</t>
+          <t xml:space="preserve">    └─ 与锈水闭环（Rustwater Loop Link） ──→ 辐射尘+赤潮孢经砂层进入卤缘与源网</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3987,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 1.3 沙豚</t>
+          <t>《瓶与源》· 1.3 沙豚</t>
         </is>
       </c>
     </row>
@@ -3488,7 +4022,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 集群迁徙（Herd Migration） ──→ Undecimber · 翻砂释放辐射尘与赤潮孢：沙豚起波井水变浊</t>
+          <t xml:space="preserve">    ├─ 集群迁徙（Herd Migration） ──→ Undecimber · 翻砂释放辐射尘与赤潮孢：沙豚起波源水变浊</t>
         </is>
       </c>
     </row>
@@ -3523,7 +4057,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 第四镜像（Fourth Mirror） ──→ 对照井兵/铁瓶/酿民：自然进化不产酒</t>
+          <t xml:space="preserve">    ├─ 第四镜像（Fourth Mirror） ──→ 对照滤兵/铁瓶/酿民：自然进化不产酒</t>
         </is>
       </c>
     </row>
@@ -3569,14 +4103,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 2.1 污染主干</t>
+          <t>《瓶与源》· 2.0 污染起因</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>官方主干 A+B+辐射尘（Canon A+B+Rad-Dust） ──→ 已定稿 · 三层污染叠加，生态酵母唯一规模化解</t>
+          <t>锈水成因链（Rustwater Causation） ──→ v8 定稿 · 先天本底+殖民并网放大+十三月时间层</t>
         </is>
       </c>
     </row>
@@ -3590,45 +4124,49 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 化学层 · 方案 A（Layer A Deep-Brine） ──→ 全年 · 深井卤层：高氯酸盐/砷/铜</t>
+          <t xml:space="preserve">    ├─ 先天层 · 星球本底（Primordial Layer） ──→ 卤缘天然有毒、嗜盐生态、弱磁辐射尘</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 生物层 · 方案 B（Layer B Red Tide） ──→ Undecimber · 嗜盐菌神经毒素，水呈铁锈红浊</t>
+          <t xml:space="preserve">    ├─ 殖民层 · 人为放大（Colonial Amplification） ──→ C.Y. 2–12 · 卤缘渠网+冷凝塔并网→源网全域锈化</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 放射层 · 辐射尘（Layer Rad-Dust） ──→ 尘暴/Undecimber · 轨道残骸+恒星风，沙海富集扬尘入水</t>
+          <t xml:space="preserve">    │       ├─ 卤缘渠网（Brine Rim Canals） ──→ C.Y. 2–8 · 沿陆海边缘截取天然卤渗出</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ Undecimber 三重峰值（Triple Peak） ──→ Undecimber · 卤压+赤潮+辐射扬尘全年最毒</t>
+          <t xml:space="preserve">    │       ├─ 冷凝塔并网（Condenser Grid Merge） ──→ C.Y. 5–10 · 卤缘卤流与冷凝水并入同一源网</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 生态酵母三重净化（Eco-Yeast Triple Purify） ──→ C.Y. 12– · 钝化毒素+包裹核素→酵母泥需处置</t>
+          <t xml:space="preserve">    │       ├─ 源流未分级（No Source Segregation） ──→ C.Y. 5–12 · 误判稀释可管理毒性</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 支渠回流污染（Branch Canal Reflux） ──→ C.Y. 8–12 · 矿冶尾液、酵母泥渗漏回流</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>支线方案 C–F（Optional C–F） ──→ 局部 · 可作区域历史诱因，非主行星主干</t>
+          <t xml:space="preserve">    └─ 时间层 · 十三月（Undecimber Layer） ──→ 每年 · 卤潮涨幅+赤潮+辐射扬尘峰值</t>
         </is>
       </c>
     </row>
@@ -3654,6 +4192,186 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 2.1 污染主干</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>官方主干 A+B+辐射尘（Canon A+B+Rad-Dust） ──→ 已定稿 · 三层污染叠加，生态酵母唯一规模化解</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 化学层 · 方案 A（Layer A Brine Rim） ──→ 全年 · 陆海卤缘天然渗出+渠网集中扩散</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 生物层 · 方案 B（Layer B Red Tide） ──→ Undecimber · 嗜盐菌沿卤缘/源网，神经毒素</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 放射层 · 辐射尘（Layer Rad-Dust） ──→ 尘暴/Undecimber · 冷凝塔、蓄源池、沙海扬尘</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ Undecimber 三重峰值（Triple Peak） ──→ Undecimber · 卤潮涨幅+赤潮+辐射扬尘</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 生态酵母三重净化（Eco-Yeast Triple Purify） ──→ C.Y. 12– · 钝化毒素+包裹核素→酵母泥需处置</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>支线方案 C–F（Optional C–F） ──→ 局部 · 支渠污染或区域历史诱因</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 2.2 垦区源网</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>垦区总水源网（Colonial Source Grid） ──→ C.Y. 2– · 非井模型 · 锈水在管网中流动分配</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 卤缘截取渠（Brine Rim Canals） ──→ C.Y. 2– · 沿陆海盆地边缘收集天然卤渗出</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 冷凝塔网（Condenser Towers） ──→ C.Y. 5– · 固陆砂岸高点集大气含水</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 蓄源池链（Reservoir Chain） ──→ C.Y. 5– · 卤缘水与冷凝水混合调蓄</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 支渠与牧场接口（Branch Canals） ──→ C.Y. 8– · 牧场矿冶酵母泥处置回流支渠</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 锈水 Rustwater ──→ 源网中一切流动储存分配的水体</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3665,7 +4383,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与井》· 2.2 十三月</t>
+          <t>《瓶与源》· 2.3 十三月</t>
         </is>
       </c>
     </row>
@@ -3707,7 +4425,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 水文峰值（Water Toxicity Peak） ──→ A+B+辐射尘 · 卤压+赤潮+沙海辐射扬尘</t>
+          <t xml:space="preserve">    ├─ 水文峰值（Water Toxicity Peak） ──→ A+B+辐射尘 · 卤潮涨幅+赤潮+沙海辐射扬尘</t>
         </is>
       </c>
     </row>
@@ -3721,7 +4439,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ C.Y. 12 井源计划植入（Wellspring Implant） ──→ C.Y. 12 · 首批净水士兵植入</t>
+          <t xml:space="preserve">    ├─ C.Y. 12 源滤计划植入（Source-Filter Implant） ──→ C.Y. 12 · 首批滤兵植入</t>
         </is>
       </c>
     </row>
@@ -3771,352 +4489,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与井》· 2.3 支线方案</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>方案 A 深井毒卤（Deep-Brine Toxicity） ──→ 推荐主干 · 高氯酸盐/砷/铜卤层，深井采水全域污染</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ Undecimber 卤压峰值（Undecimber Brine Peak） ──→ 每年 · 地下卤层渗透率年度最高</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>方案 B 流浪赤潮（Wandering Red Tide） ──→ 推荐叠加 · 本土嗜盐菌季节性神经毒素</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 赤潮高峰（Red Tide Peak） ──→ Undecimber · 全年水质最差月份</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>方案 C terraform 遗产（Terraform Legacy） ──→ 可选 · 早期大气改造站催化剂泄漏</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>方案 D 矿冶尾液（Smelting Tailings） ──→ 可选 · 机甲燃料炼矿尾液渗入含水层</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>方案 E 化武残留（Chemical War Residue） ──→ 可选 · 殖民内战化学剂污染流域</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>方案 F 尘暴带电粒子（Dust Storm Ions） ──→ 可选 · 双恒星尘暴金属微粒随雨入水</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="7" t="inlineStr"/>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>推荐组合 A+B（Recommended A+B） ──→ 已并入主干 · 见「污染官方主干」模块</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="7" t="inlineStr"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>生态酵母（统一应答）（Eco-Yeast Response） ──→ C.Y. 12– · 所有方案共同技术解：锈水→生态酿</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A16:C16"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与井》· 3.1 生态酵母</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>生态酵母（基础株）（Saccharomyces vitae） ──→ C.Y. 12– · 三重净化：化学毒+生物毒+辐射尘</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ W-Strain（W-Strain (Military)） ──→ C.Y. 12–17 · 军用稳态型</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │   │</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │       └─ 井源计划（Wellspring Program） ──→ C.Y. 12–17 · 第一批植入者为净水超级士兵</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │           │</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │           └─ 净水士兵（井兵）（Aqua-Soldiers） ──→ C.Y. 12–17 · 锈水→内源生态酿 2–4%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │               │</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │               └─ 井醒（Well-Awake） ──→ C.Y. 37+ · W-Strain 残留 / 幸存井兵</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ R-Strain（R-Strain (Civilian)） ──→ C.Y. 12– · 民用救灾型</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │   │</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │       └─ 生态酿（Eco-Brew） ──→ C.Y. 12– · 2–4%，公开合法，社会认知「酵母=希望」</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ F-Strain（F-Strain (Fuel)） ──→ C.Y. 15– · 燃料高产型</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        ├─ 活燃料计划（Living Fuel Program） ──→ C.Y. 15–23 · 人体活体发酵容器</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        │   │</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        │       └─ 醇民 Gen-0（Brewfolk Gen-0） ──→ C.Y. 15–23 · 血肉容器，已基本灭绝</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        └─ 铁瓶计划（Synth-Bottle Program） ──→ C.Y. 23–30 · 菌株移植至机械载体</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                ├─ 铁瓶 Gen-1（Synth-Bottle Gen-1） ──→ C.Y. 23– · 无意识机械产力，圈养/野生</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                │   │</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">            │       └─ 瓶醒（Synth-Awake） ──→ C.Y. 37+ · F-Strain 网络共振，集体性觉醒</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">                └─ 酿民 Gen-2（Brewfolk Gen-2） ──→ C.Y. 37+ · 觉醒意识体，冲突中心</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A16:C16"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200347) from my-cloud-project@d6e01df
</commit_message>
<xml_diff>
--- a/瓶与井世界观树状图.xlsx
+++ b/瓶与井世界观树状图.xlsx
@@ -21,9 +21,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. 威士忌经济" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7b. 城带与荒原" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. 势力格局" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. 叙事入口" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. 锈钉" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 锈钉开篇" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. 戒酒教" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. 叙事入口" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. 锈钉" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 锈钉开篇" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -496,7 +497,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-20-v15</t>
+          <t>2026-07-20-v16</t>
         </is>
       </c>
     </row>
@@ -799,26 +800,33 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  13. 9. 叙事入口</t>
+          <t xml:space="preserve">  13. 8b. 戒酒教</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  14. 10. 锈钉</t>
+          <t xml:space="preserve">  14. 9. 叙事入口</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  15. 11. 锈钉开篇</t>
+          <t xml:space="preserve">  15. 10. 锈钉</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  16. 11. 锈钉开篇</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="B7:C7"/>
@@ -832,6 +840,7 @@
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A42:C42"/>
     <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A47:C47"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A32:C32"/>
     <mergeCell ref="A14:C14"/>
@@ -1383,7 +1392,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1461,58 +1470,217 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 收割派/纯净派</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 反身作酒窖 · 分裂两派 · 见模块7b</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
+      <c r="A16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 收割派（Harvest Faction） ──→ C.Y. 42 · 取酵不取命 · 灵魂可赎</t>
+          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 8b. 戒酒教</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 起源于胃植入/酵母宗教化 · 禁饮威士忌</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 共同基底（Shared Creed） ──→ 肉体不得为酒窖 · 不隶属城酿署</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿与荒原非法提取并存</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>收割派 Reapers（Harvest Faction） ──→ C.Y. 42 · 酵可赎命不可夺 · 反击晕非法提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 击晕提取即渎 · 城带采酿为契约束缚</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 赎酵站（Redemption Still） ──→ 锈水去毒发酵 · 不取自酿民体内</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 庇护廊（Shelter Corridors） ──→ 收留觉醒逃亡酿民 · 城缘地下</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 赎酵礼（Redemption Rite） ──→ 伏击猎人求放人/少取 · 不追杀客户</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 城缘灰诊（Rim Clinics） ──→ 卖去毒锈水 · 治提取后遗症 · 换情报</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可谈判赎人 · 「可赎之渎」档案</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>纯净派 Purifiers（Purity Faction） ──→ C.Y. 42 · 酒即秽瓶即牢 · 凡酿皆罪</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 纯净派（Purity Faction） ──→ C.Y. 42 · 威士忌即罪恶 · 焚毁铁瓶酿民</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="7" t="inlineStr"/>
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 否定城带/黑市/铁瓶生态群 · 发酵舱须净化</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人</t>
+          <t xml:space="preserve">    ├─ 尘骑巡游（Dust Riders） ──→ 铁瓶线/Saloon机动 · 十三月尘暴掩护</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="7" t="inlineStr"/>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 净火行动（Purifying Fire） ──→ 焚回收槽 · 黑市酵舱 · 铁瓶外露发酵舱</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>酒镇 Saloon ──→ C.Y. 42 · 中立 · 劣酿 · 悬赏 · 情报</t>
+          <t xml:space="preserve">    ├─ 断酿伏击（Sever Brew Ambush） ──→ 袭击猎人交货点 · 砸酵管放目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 净居聚落（Ascetic Communes） ──→ 荒漠深处 · 只饮去毒无醇锈水</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 净化目标 · 与收割派互斥</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="23">
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A22:C22"/>
@@ -1524,6 +1692,7 @@
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A6:C6"/>
@@ -1534,7 +1703,115 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 9. 叙事入口</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教收割派（Temperance Reapers） ──→ C.Y. 42 · 赎酵站/庇护廊 · 反非法提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教纯净派（Temperance Purifiers） ──→ C.Y. 42 · 尘骑净火 · 焚黑市与铁瓶外露舱</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1550,54 +1827,70 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与源》· 9. 叙事入口</t>
+          <t>《瓶与源》· 10. 锈钉</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr"/>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
+          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr"/>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
+          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr"/>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
+          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
+          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
         </is>
       </c>
     </row>
@@ -1618,107 +1911,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与源》· 10. 锈钉</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1808,7 +2001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C185"/>
+  <dimension ref="A1:C208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -2717,241 +2910,386 @@
     <row r="147" outlineLevel="1" ht="16" customHeight="1">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 收割派/纯净派</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 反身作酒窖 · 分裂两派 · 见模块7b</t>
         </is>
       </c>
     </row>
     <row r="148" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A148" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
+      <c r="A148" s="7" t="inlineStr"/>
     </row>
     <row r="149" outlineLevel="1" ht="16" customHeight="1">
       <c r="A149" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 收割派（Harvest Faction） ──→ C.Y. 42 · 取酵不取命 · 灵魂可赎</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A150" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 纯净派（Purity Faction） ──→ C.Y. 42 · 威士忌即罪恶 · 焚毁铁瓶酿民</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A151" s="7" t="inlineStr"/>
+          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>▸ 8b. 戒酒教</t>
+        </is>
+      </c>
     </row>
     <row r="152" outlineLevel="1" ht="16" customHeight="1">
       <c r="A152" s="7" t="inlineStr">
         <is>
-          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 起源于胃植入/酵母宗教化 · 禁饮威士忌</t>
         </is>
       </c>
     </row>
     <row r="153" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A153" s="7" t="inlineStr"/>
+      <c r="A153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="154" outlineLevel="1" ht="16" customHeight="1">
       <c r="A154" s="7" t="inlineStr">
         <is>
-          <t>酒镇 Saloon ──→ C.Y. 42 · 中立 · 劣酿 · 悬赏 · 情报</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="6" t="inlineStr">
-        <is>
-          <t>▸ 9. 叙事入口</t>
-        </is>
-      </c>
+          <t xml:space="preserve">    ├─ 共同基底（Shared Creed） ──→ 肉体不得为酒窖 · 不隶属城酿署</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A155" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿与荒原非法提取并存</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A156" s="7" t="inlineStr"/>
     </row>
     <row r="157" outlineLevel="1" ht="16" customHeight="1">
       <c r="A157" s="7" t="inlineStr">
         <is>
-          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+          <t>收割派 Reapers（Harvest Faction） ──→ C.Y. 42 · 酵可赎命不可夺 · 反击晕非法提取</t>
         </is>
       </c>
     </row>
     <row r="158" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A158" s="7" t="inlineStr"/>
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="159" outlineLevel="1" ht="16" customHeight="1">
       <c r="A159" s="7" t="inlineStr">
         <is>
-          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 击晕提取即渎 · 城带采酿为契约束缚</t>
         </is>
       </c>
     </row>
     <row r="160" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A160" s="7" t="inlineStr"/>
+      <c r="A160" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 赎酵站（Redemption Still） ──→ 锈水去毒发酵 · 不取自酿民体内</t>
+        </is>
+      </c>
     </row>
     <row r="161" outlineLevel="1" ht="16" customHeight="1">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
+          <t xml:space="preserve">    ├─ 庇护廊（Shelter Corridors） ──→ 收留觉醒逃亡酿民 · 城缘地下</t>
         </is>
       </c>
     </row>
     <row r="162" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A162" s="7" t="inlineStr"/>
+      <c r="A162" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 赎酵礼（Redemption Rite） ──→ 伏击猎人求放人/少取 · 不追杀客户</t>
+        </is>
+      </c>
     </row>
     <row r="163" outlineLevel="1" ht="16" customHeight="1">
       <c r="A163" s="7" t="inlineStr">
         <is>
-          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
+          <t xml:space="preserve">    ├─ 城缘灰诊（Rim Clinics） ──→ 卖去毒锈水 · 治提取后遗症 · 换情报</t>
         </is>
       </c>
     </row>
     <row r="164" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A164" s="7" t="inlineStr"/>
+      <c r="A164" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可谈判赎人 · 「可赎之渎」档案</t>
+        </is>
+      </c>
     </row>
     <row r="165" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A165" s="7" t="inlineStr">
-        <is>
-          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="6" t="inlineStr">
-        <is>
-          <t>▸ 10. 锈钉</t>
+      <c r="A165" s="7" t="inlineStr"/>
+    </row>
+    <row r="166" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A166" s="7" t="inlineStr">
+        <is>
+          <t>纯净派 Purifiers（Purity Faction） ──→ C.Y. 42 · 酒即秽瓶即牢 · 凡酿皆罪</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="168" outlineLevel="1" ht="16" customHeight="1">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 否定城带/黑市/铁瓶生态群 · 发酵舱须净化</t>
         </is>
       </c>
     </row>
     <row r="169" outlineLevel="1" ht="16" customHeight="1">
       <c r="A169" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 尘骑巡游（Dust Riders） ──→ 铁瓶线/Saloon机动 · 十三月尘暴掩护</t>
         </is>
       </c>
     </row>
     <row r="170" outlineLevel="1" ht="16" customHeight="1">
       <c r="A170" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
+          <t xml:space="preserve">    ├─ 净火行动（Purifying Fire） ──→ 焚回收槽 · 黑市酵舱 · 铁瓶外露发酵舱</t>
         </is>
       </c>
     </row>
     <row r="171" outlineLevel="1" ht="16" customHeight="1">
       <c r="A171" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
+          <t xml:space="preserve">    ├─ 断酿伏击（Sever Brew Ambush） ──→ 袭击猎人交货点 · 砸酵管放目标</t>
         </is>
       </c>
     </row>
     <row r="172" outlineLevel="1" ht="16" customHeight="1">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
+          <t xml:space="preserve">    ├─ 净居聚落（Ascetic Communes） ──→ 荒漠深处 · 只饮去毒无醇锈水</t>
         </is>
       </c>
     </row>
     <row r="173" outlineLevel="1" ht="16" customHeight="1">
       <c r="A173" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
-        </is>
-      </c>
-    </row>
-    <row r="174" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A174" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
-        </is>
-      </c>
-    </row>
-    <row r="175" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A175" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 净化目标 · 与收割派互斥</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>▸ 9. 叙事入口</t>
         </is>
       </c>
     </row>
     <row r="176" outlineLevel="1" ht="16" customHeight="1">
       <c r="A176" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="6" t="inlineStr">
-        <is>
-          <t>▸ 11. 锈钉开篇</t>
+          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A177" s="7" t="inlineStr"/>
+    </row>
+    <row r="178" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A178" s="7" t="inlineStr">
+        <is>
+          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
         </is>
       </c>
     </row>
     <row r="179" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A179" s="7" t="inlineStr">
-        <is>
-          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 非法提取链</t>
-        </is>
-      </c>
+      <c r="A179" s="7" t="inlineStr"/>
     </row>
     <row r="180" outlineLevel="1" ht="16" customHeight="1">
       <c r="A180" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
         </is>
       </c>
     </row>
     <row r="181" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A181" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七提取委托 ×5</t>
-        </is>
-      </c>
+      <c r="A181" s="7" t="inlineStr"/>
     </row>
     <row r="182" outlineLevel="1" ht="16" customHeight="1">
       <c r="A182" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
+          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
         </is>
       </c>
     </row>
     <row r="183" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A183" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
-        </is>
-      </c>
+      <c r="A183" s="7" t="inlineStr"/>
     </row>
     <row r="184" outlineLevel="1" ht="16" customHeight="1">
       <c r="A184" s="7" t="inlineStr">
         <is>
+          <t>戒酒教收割派（Temperance Reapers） ──→ C.Y. 42 · 赎酵站/庇护廊 · 反非法提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A185" s="7" t="inlineStr"/>
+    </row>
+    <row r="186" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A186" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教纯净派（Temperance Purifiers） ──→ C.Y. 42 · 尘骑净火 · 焚黑市与铁瓶外露舱</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A187" s="7" t="inlineStr"/>
+    </row>
+    <row r="188" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A188" s="7" t="inlineStr">
+        <is>
+          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>▸ 10. 锈钉</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A191" s="7" t="inlineStr">
+        <is>
+          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A198" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="6" t="inlineStr">
+        <is>
+          <t>▸ 11. 锈钉开篇</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A202" s="7" t="inlineStr">
+        <is>
+          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 非法提取链</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七提取委托 ×5</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A207" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
         </is>
       </c>
     </row>
-    <row r="185" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A185" s="7" t="inlineStr">
+    <row r="208" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A208" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">    └─ 背景侧写（Metro Contrast） ──→ 合法采酿行情 vs 黑市提取价</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="170">
+  <mergeCells count="192">
     <mergeCell ref="A128:C128"/>
+    <mergeCell ref="A193:C193"/>
     <mergeCell ref="A80:C80"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A208:C208"/>
     <mergeCell ref="A89:C89"/>
     <mergeCell ref="A136:C136"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A105:C105"/>
+    <mergeCell ref="A192:C192"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A57:C57"/>
     <mergeCell ref="A113:C113"/>
@@ -2959,6 +3297,7 @@
     <mergeCell ref="A71:C71"/>
     <mergeCell ref="A185:C185"/>
     <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A194:C194"/>
     <mergeCell ref="A181:C181"/>
     <mergeCell ref="A91:C91"/>
     <mergeCell ref="A184:C184"/>
@@ -2968,6 +3307,7 @@
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="A165:C165"/>
     <mergeCell ref="A63:C63"/>
+    <mergeCell ref="A155:C155"/>
     <mergeCell ref="A93:C93"/>
     <mergeCell ref="A173:C173"/>
     <mergeCell ref="A130:C130"/>
@@ -2983,11 +3323,13 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A119:C119"/>
     <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A174:C174"/>
+    <mergeCell ref="A196:C196"/>
+    <mergeCell ref="A205:C205"/>
     <mergeCell ref="A183:C183"/>
     <mergeCell ref="A66:C66"/>
     <mergeCell ref="A118:C118"/>
     <mergeCell ref="A75:C75"/>
+    <mergeCell ref="A198:C198"/>
     <mergeCell ref="A120:C120"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="A12:C12"/>
@@ -3012,18 +3354,23 @@
     <mergeCell ref="A170:C170"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A202:C202"/>
     <mergeCell ref="A58:C58"/>
     <mergeCell ref="A67:C67"/>
     <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A186:C186"/>
     <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A201:C201"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A60:C60"/>
     <mergeCell ref="A123:C123"/>
+    <mergeCell ref="A197:C197"/>
     <mergeCell ref="A146:C146"/>
     <mergeCell ref="A124:C124"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A172:C172"/>
     <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A187:C187"/>
     <mergeCell ref="A99:C99"/>
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A108:C108"/>
@@ -3035,21 +3382,25 @@
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A86:C86"/>
+    <mergeCell ref="A204:C204"/>
     <mergeCell ref="A42:C42"/>
     <mergeCell ref="A151:C151"/>
     <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A188:C188"/>
     <mergeCell ref="A126:C126"/>
     <mergeCell ref="A141:C141"/>
     <mergeCell ref="A135:C135"/>
-    <mergeCell ref="A150:C150"/>
+    <mergeCell ref="A206:C206"/>
     <mergeCell ref="A62:C62"/>
     <mergeCell ref="A144:C144"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A125:C125"/>
+    <mergeCell ref="A190:C190"/>
     <mergeCell ref="A72:C72"/>
     <mergeCell ref="A134:C134"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A112:C112"/>
+    <mergeCell ref="A199:C199"/>
     <mergeCell ref="A152:C152"/>
     <mergeCell ref="A127:C127"/>
     <mergeCell ref="A167:C167"/>
@@ -3060,6 +3411,7 @@
     <mergeCell ref="A182:C182"/>
     <mergeCell ref="A64:C64"/>
     <mergeCell ref="A98:C98"/>
+    <mergeCell ref="A191:C191"/>
     <mergeCell ref="A169:C169"/>
     <mergeCell ref="A107:C107"/>
     <mergeCell ref="A178:C178"/>
@@ -3070,6 +3422,7 @@
     <mergeCell ref="A162:C162"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="A137:C137"/>
+    <mergeCell ref="A177:C177"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A90:C90"/>
     <mergeCell ref="A164:C164"/>
@@ -3080,8 +3433,10 @@
     <mergeCell ref="A139:C139"/>
     <mergeCell ref="A154:C154"/>
     <mergeCell ref="A129:C129"/>
+    <mergeCell ref="A195:C195"/>
     <mergeCell ref="A76:C76"/>
     <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A203:C203"/>
     <mergeCell ref="A85:C85"/>
     <mergeCell ref="A116:C116"/>
     <mergeCell ref="A8:C8"/>
@@ -3102,10 +3457,12 @@
     <mergeCell ref="A143:C143"/>
     <mergeCell ref="A92:C92"/>
     <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A166:C166"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="A142:C142"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A207:C207"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A94:C94"/>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200351) from my-cloud-project@73d5280
</commit_message>
<xml_diff>
--- a/瓶与井世界观树状图.xlsx
+++ b/瓶与井世界观树状图.xlsx
@@ -497,7 +497,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-20-v16</t>
+          <t>2026-07-20-v17</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 反身作酒窖 · 分裂两派 · 见模块7b</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 与酿民敌对 · 完全摒弃/圣火 · 见8b</t>
         </is>
       </c>
     </row>
@@ -1480,7 +1480,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人</t>
+          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人与戒酒教</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1530,7 +1530,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 起源于胃植入/酵母宗教化 · 禁饮威士忌</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 酿民即秽种 · 与酿民敌对 · 教团分裂</t>
         </is>
       </c>
     </row>
@@ -1544,14 +1544,14 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 共同基底（Shared Creed） ──→ 肉体不得为酒窖 · 不隶属城酿署</t>
+          <t xml:space="preserve">    ├─ 共同教义（Shared Creed） ──→ 不庇护酿民 · 禁饮体内威士忌</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿与荒原非法提取并存</t>
+          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿后 · 处置秽种路线之争</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>收割派 Reapers（Harvest Faction） ──→ C.Y. 42 · 酵可赎命不可夺 · 反击晕非法提取</t>
+          <t>完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼温和 · 用泉不用窖</t>
         </is>
       </c>
     </row>
@@ -1575,115 +1575,84 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 击晕提取即渎 · 城带采酿为契约束缚</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 利用离体酵母锈水 · 完全摒弃酿民</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 赎酵站（Redemption Still） ──→ 锈水去毒发酵 · 不取自酿民体内</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 隔离/诱捕移交/告密 · 不亲手焚杀</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 庇护廊（Shelter Corridors） ──→ 收留觉醒逃亡酿民 · 城缘地下</t>
+          <t xml:space="preserve">    ├─ 净泉聚落（Pure Spring Communes） ──→ 离体培菌去毒 · 卖洁净锈水</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 赎酵礼（Redemption Rite） ──→ 伏击猎人求放人/少取 · 不追杀客户</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可付情报费借猎人刀</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 城缘灰诊（Rim Clinics） ──→ 卖去毒锈水 · 治提取后遗症 · 换情报</t>
-        </is>
-      </c>
+      <c r="A14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可谈判赎人 · 「可赎之渎」档案</t>
+          <t>圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼极端 · 秽须焚</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr"/>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>纯净派 Purifiers（Purity Faction） ──→ C.Y. 42 · 酒即秽瓶即牢 · 凡酿皆罪</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 酿民须圣火净化 · 不留窖芯</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 焚杀酿民/回收槽/铁瓶外露舱</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 否定城带/黑市/铁瓶生态群 · 发酵舱须净化</t>
+          <t xml:space="preserve">    ├─ 尘骑殉火（Dust Riders） ──→ 机动圣战 · 十三月尘暴掩护</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 尘骑巡游（Dust Riders） ──→ 铁瓶线/Saloon机动 · 十三月尘暴掩护</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 净火行动（Purifying Fire） ──→ 焚回收槽 · 黑市酵舱 · 铁瓶外露发酵舱</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 断酿伏击（Sever Brew Ambush） ──→ 袭击猎人交货点 · 砸酵管放目标</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 净居聚落（Ascetic Communes） ──→ 荒漠深处 · 只饮去毒无醇锈水</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 净化目标 · 与收割派互斥</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 必杀 · 提取手与秽种同焚</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="19">
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A20:C20"/>
@@ -1692,7 +1661,6 @@
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A6:C6"/>
@@ -1766,7 +1734,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>戒酒教收割派（Temperance Reapers） ──→ C.Y. 42 · 赎酵站/庇护廊 · 反非法提取</t>
+          <t>戒酒教完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼 · 用泉不用窖 · 隔离诱捕酿民</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1744,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>戒酒教纯净派（Temperance Purifiers） ──→ C.Y. 42 · 尘骑净火 · 焚黑市与铁瓶外露舱</t>
+          <t>戒酒教圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼 · 秽须焚 · 焚杀酿民</t>
         </is>
       </c>
     </row>
@@ -2001,7 +1969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C208"/>
+  <dimension ref="A1:C204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -2910,7 +2878,7 @@
     <row r="147" outlineLevel="1" ht="16" customHeight="1">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 反身作酒窖 · 分裂两派 · 见模块7b</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 与酿民敌对 · 完全摒弃/圣火 · 见8b</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2888,7 @@
     <row r="149" outlineLevel="1" ht="16" customHeight="1">
       <c r="A149" s="7" t="inlineStr">
         <is>
-          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人</t>
+          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人与戒酒教</t>
         </is>
       </c>
     </row>
@@ -2934,7 +2902,7 @@
     <row r="152" outlineLevel="1" ht="16" customHeight="1">
       <c r="A152" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 起源于胃植入/酵母宗教化 · 禁饮威士忌</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 酿民即秽种 · 与酿民敌对 · 教团分裂</t>
         </is>
       </c>
     </row>
@@ -2948,14 +2916,14 @@
     <row r="154" outlineLevel="1" ht="16" customHeight="1">
       <c r="A154" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 共同基底（Shared Creed） ──→ 肉体不得为酒窖 · 不隶属城酿署</t>
+          <t xml:space="preserve">    ├─ 共同教义（Shared Creed） ──→ 不庇护酿民 · 禁饮体内威士忌</t>
         </is>
       </c>
     </row>
     <row r="155" outlineLevel="1" ht="16" customHeight="1">
       <c r="A155" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿与荒原非法提取并存</t>
+          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿后 · 处置秽种路线之争</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2933,7 @@
     <row r="157" outlineLevel="1" ht="16" customHeight="1">
       <c r="A157" s="7" t="inlineStr">
         <is>
-          <t>收割派 Reapers（Harvest Faction） ──→ C.Y. 42 · 酵可赎命不可夺 · 反击晕非法提取</t>
+          <t>完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼温和 · 用泉不用窖</t>
         </is>
       </c>
     </row>
@@ -2979,115 +2947,107 @@
     <row r="159" outlineLevel="1" ht="16" customHeight="1">
       <c r="A159" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 击晕提取即渎 · 城带采酿为契约束缚</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 利用离体酵母锈水 · 完全摒弃酿民</t>
         </is>
       </c>
     </row>
     <row r="160" outlineLevel="1" ht="16" customHeight="1">
       <c r="A160" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 赎酵站（Redemption Still） ──→ 锈水去毒发酵 · 不取自酿民体内</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 隔离/诱捕移交/告密 · 不亲手焚杀</t>
         </is>
       </c>
     </row>
     <row r="161" outlineLevel="1" ht="16" customHeight="1">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 庇护廊（Shelter Corridors） ──→ 收留觉醒逃亡酿民 · 城缘地下</t>
+          <t xml:space="preserve">    ├─ 净泉聚落（Pure Spring Communes） ──→ 离体培菌去毒 · 卖洁净锈水</t>
         </is>
       </c>
     </row>
     <row r="162" outlineLevel="1" ht="16" customHeight="1">
       <c r="A162" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 赎酵礼（Redemption Rite） ──→ 伏击猎人求放人/少取 · 不追杀客户</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可付情报费借猎人刀</t>
         </is>
       </c>
     </row>
     <row r="163" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A163" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 城缘灰诊（Rim Clinics） ──→ 卖去毒锈水 · 治提取后遗症 · 换情报</t>
-        </is>
-      </c>
+      <c r="A163" s="7" t="inlineStr"/>
     </row>
     <row r="164" outlineLevel="1" ht="16" customHeight="1">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可谈判赎人 · 「可赎之渎」档案</t>
+          <t>圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼极端 · 秽须焚</t>
         </is>
       </c>
     </row>
     <row r="165" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A165" s="7" t="inlineStr"/>
+      <c r="A165" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="166" outlineLevel="1" ht="16" customHeight="1">
       <c r="A166" s="7" t="inlineStr">
         <is>
-          <t>纯净派 Purifiers（Purity Faction） ──→ C.Y. 42 · 酒即秽瓶即牢 · 凡酿皆罪</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 酿民须圣火净化 · 不留窖芯</t>
         </is>
       </c>
     </row>
     <row r="167" outlineLevel="1" ht="16" customHeight="1">
       <c r="A167" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 焚杀酿民/回收槽/铁瓶外露舱</t>
         </is>
       </c>
     </row>
     <row r="168" outlineLevel="1" ht="16" customHeight="1">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 否定城带/黑市/铁瓶生态群 · 发酵舱须净化</t>
+          <t xml:space="preserve">    ├─ 尘骑殉火（Dust Riders） ──→ 机动圣战 · 十三月尘暴掩护</t>
         </is>
       </c>
     </row>
     <row r="169" outlineLevel="1" ht="16" customHeight="1">
       <c r="A169" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 尘骑巡游（Dust Riders） ──→ 铁瓶线/Saloon机动 · 十三月尘暴掩护</t>
-        </is>
-      </c>
-    </row>
-    <row r="170" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A170" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 净火行动（Purifying Fire） ──→ 焚回收槽 · 黑市酵舱 · 铁瓶外露发酵舱</t>
-        </is>
-      </c>
-    </row>
-    <row r="171" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A171" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 断酿伏击（Sever Brew Ambush） ──→ 袭击猎人交货点 · 砸酵管放目标</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 必杀 · 提取手与秽种同焚</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>▸ 9. 叙事入口</t>
         </is>
       </c>
     </row>
     <row r="172" outlineLevel="1" ht="16" customHeight="1">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 净居聚落（Ascetic Communes） ──→ 荒漠深处 · 只饮去毒无醇锈水</t>
+          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
         </is>
       </c>
     </row>
     <row r="173" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A173" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 净化目标 · 与收割派互斥</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="6" t="inlineStr">
-        <is>
-          <t>▸ 9. 叙事入口</t>
-        </is>
-      </c>
+      <c r="A173" s="7" t="inlineStr"/>
+    </row>
+    <row r="174" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A174" s="7" t="inlineStr">
+        <is>
+          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A175" s="7" t="inlineStr"/>
     </row>
     <row r="176" outlineLevel="1" ht="16" customHeight="1">
       <c r="A176" s="7" t="inlineStr">
         <is>
-          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3057,7 @@
     <row r="178" outlineLevel="1" ht="16" customHeight="1">
       <c r="A178" s="7" t="inlineStr">
         <is>
-          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
+          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3067,7 @@
     <row r="180" outlineLevel="1" ht="16" customHeight="1">
       <c r="A180" s="7" t="inlineStr">
         <is>
-          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
+          <t>戒酒教完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼 · 用泉不用窖 · 隔离诱捕酿民</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3077,7 @@
     <row r="182" outlineLevel="1" ht="16" customHeight="1">
       <c r="A182" s="7" t="inlineStr">
         <is>
-          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
+          <t>戒酒教圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼 · 秽须焚 · 焚杀酿民</t>
         </is>
       </c>
     </row>
@@ -3127,164 +3087,143 @@
     <row r="184" outlineLevel="1" ht="16" customHeight="1">
       <c r="A184" s="7" t="inlineStr">
         <is>
-          <t>戒酒教收割派（Temperance Reapers） ──→ C.Y. 42 · 赎酵站/庇护廊 · 反非法提取</t>
-        </is>
-      </c>
-    </row>
-    <row r="185" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A185" s="7" t="inlineStr"/>
-    </row>
-    <row r="186" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A186" s="7" t="inlineStr">
-        <is>
-          <t>戒酒教纯净派（Temperance Purifiers） ──→ C.Y. 42 · 尘骑净火 · 焚黑市与铁瓶外露舱</t>
+          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="6" t="inlineStr">
+        <is>
+          <t>▸ 10. 锈钉</t>
         </is>
       </c>
     </row>
     <row r="187" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A187" s="7" t="inlineStr"/>
+      <c r="A187" s="7" t="inlineStr">
+        <is>
+          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
+        </is>
+      </c>
     </row>
     <row r="188" outlineLevel="1" ht="16" customHeight="1">
       <c r="A188" s="7" t="inlineStr">
         <is>
-          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="6" t="inlineStr">
-        <is>
-          <t>▸ 10. 锈钉</t>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A189" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
         </is>
       </c>
     </row>
     <row r="191" outlineLevel="1" ht="16" customHeight="1">
       <c r="A191" s="7" t="inlineStr">
         <is>
-          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
+          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
         </is>
       </c>
     </row>
     <row r="192" outlineLevel="1" ht="16" customHeight="1">
       <c r="A192" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
         </is>
       </c>
     </row>
     <row r="193" outlineLevel="1" ht="16" customHeight="1">
       <c r="A193" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
+          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
         </is>
       </c>
     </row>
     <row r="194" outlineLevel="1" ht="16" customHeight="1">
       <c r="A194" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
+          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
         </is>
       </c>
     </row>
     <row r="195" outlineLevel="1" ht="16" customHeight="1">
       <c r="A195" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
-        </is>
-      </c>
-    </row>
-    <row r="196" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A196" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
-        </is>
-      </c>
-    </row>
-    <row r="197" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A197" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
+          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="6" t="inlineStr">
+        <is>
+          <t>▸ 11. 锈钉开篇</t>
         </is>
       </c>
     </row>
     <row r="198" outlineLevel="1" ht="16" customHeight="1">
       <c r="A198" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
+          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 非法提取链</t>
         </is>
       </c>
     </row>
     <row r="199" outlineLevel="1" ht="16" customHeight="1">
       <c r="A199" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="6" t="inlineStr">
-        <is>
-          <t>▸ 11. 锈钉开篇</t>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七提取委托 ×5</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
         </is>
       </c>
     </row>
     <row r="202" outlineLevel="1" ht="16" customHeight="1">
       <c r="A202" s="7" t="inlineStr">
         <is>
-          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 非法提取链</t>
+          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
         </is>
       </c>
     </row>
     <row r="203" outlineLevel="1" ht="16" customHeight="1">
       <c r="A203" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
         </is>
       </c>
     </row>
     <row r="204" outlineLevel="1" ht="16" customHeight="1">
       <c r="A204" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七提取委托 ×5</t>
-        </is>
-      </c>
-    </row>
-    <row r="205" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A205" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
-        </is>
-      </c>
-    </row>
-    <row r="206" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A206" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
-        </is>
-      </c>
-    </row>
-    <row r="207" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A207" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
-        </is>
-      </c>
-    </row>
-    <row r="208" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A208" s="7" t="inlineStr">
-        <is>
           <t xml:space="preserve">    └─ 背景侧写（Metro Contrast） ──→ 合法采酿行情 vs 黑市提取价</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="192">
+  <mergeCells count="188">
     <mergeCell ref="A128:C128"/>
     <mergeCell ref="A193:C193"/>
     <mergeCell ref="A80:C80"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A208:C208"/>
     <mergeCell ref="A89:C89"/>
     <mergeCell ref="A136:C136"/>
     <mergeCell ref="A21:C21"/>
@@ -3295,7 +3234,6 @@
     <mergeCell ref="A113:C113"/>
     <mergeCell ref="A179:C179"/>
     <mergeCell ref="A71:C71"/>
-    <mergeCell ref="A185:C185"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A194:C194"/>
     <mergeCell ref="A181:C181"/>
@@ -3323,8 +3261,7 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A119:C119"/>
     <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A196:C196"/>
-    <mergeCell ref="A205:C205"/>
+    <mergeCell ref="A174:C174"/>
     <mergeCell ref="A183:C183"/>
     <mergeCell ref="A66:C66"/>
     <mergeCell ref="A118:C118"/>
@@ -3344,6 +3281,7 @@
     <mergeCell ref="A106:C106"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A200:C200"/>
     <mergeCell ref="A81:C81"/>
     <mergeCell ref="A38:C38"/>
     <mergeCell ref="A96:C96"/>
@@ -3351,7 +3289,6 @@
     <mergeCell ref="A121:C121"/>
     <mergeCell ref="A161:C161"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A170:C170"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A202:C202"/>
@@ -3380,6 +3317,7 @@
     <mergeCell ref="A163:C163"/>
     <mergeCell ref="A158:C158"/>
     <mergeCell ref="A101:C101"/>
+    <mergeCell ref="A189:C189"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A86:C86"/>
     <mergeCell ref="A204:C204"/>
@@ -3390,7 +3328,6 @@
     <mergeCell ref="A126:C126"/>
     <mergeCell ref="A141:C141"/>
     <mergeCell ref="A135:C135"/>
-    <mergeCell ref="A206:C206"/>
     <mergeCell ref="A62:C62"/>
     <mergeCell ref="A144:C144"/>
     <mergeCell ref="A20:C20"/>
@@ -3462,7 +3399,6 @@
     <mergeCell ref="A142:C142"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A207:C207"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A94:C94"/>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200413) from my-cloud-project@9f560ad
</commit_message>
<xml_diff>
--- a/瓶与井世界观树状图.xlsx
+++ b/瓶与井世界观树状图.xlsx
@@ -21,10 +21,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. 威士忌经济" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7b. 城带与荒原" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. 势力格局" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. 戒酒教" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. 叙事入口" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. 锈钉" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 锈钉开篇" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8a. 当地警署" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8c. 酿造帮" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. 戒酒教" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. 叙事入口" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. 锈钉" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 锈钉开篇" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -660,7 +662,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【第三批】囚犯放逐 · 威士忌分级 · 名义猎人/实质非法提取</t>
+          <t xml:space="preserve">    ├─ 【第三批】囚犯放逐 · 威士忌分级 · 警署悬赏/实质非法提取</t>
         </is>
       </c>
     </row>
@@ -674,7 +676,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【城带】二代酿民合法采酿 · 琥珀交易所</t>
+          <t xml:space="preserve">    ├─ 【城带】二代酿民合法采酿 · 琥珀交易所 · 当地警署</t>
         </is>
       </c>
     </row>
@@ -688,7 +690,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 【荒原】击晕提取委托 · 黑市出货 · 锈钉行尸走肉循环</t>
+          <t xml:space="preserve">    ├─ 【荒原】警署悬赏 · 酿造帮园区 · 黑市出货 · 锈钉行尸走肉循环</t>
         </is>
       </c>
     </row>
@@ -800,33 +802,47 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  13. 8b. 戒酒教</t>
+          <t xml:space="preserve">  13. 8a. 当地警署</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  14. 9. 叙事入口</t>
+          <t xml:space="preserve">  14. 8c. 酿造帮</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  15. 10. 锈钉</t>
+          <t xml:space="preserve">  15. 8b. 戒酒教</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  16. 11. 锈钉开篇</t>
+          <t xml:space="preserve">  16. 9. 叙事入口</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  17. 10. 锈钉</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  18. 11. 锈钉开篇</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="45">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="B7:C7"/>
@@ -861,10 +877,12 @@
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A48:C48"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B5:C5"/>
@@ -940,7 +958,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 赏金猎人（The Hunter） ──→ C.Y. 30– · 名义追捕 · 实质击晕提取售黑市</t>
+          <t xml:space="preserve">    └─ 缉拿手（The Hunter） ──→ C.Y. 30– · 警署悬赏承包商 · 实质击晕提取售黑市</t>
         </is>
       </c>
     </row>
@@ -964,7 +982,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1103,43 +1121,50 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 荒原逃亡/未登记（Wasteland Fugitive） ──→ C.Y. 42 · 脱离群落或从未登记 · 提取委托常见目标</t>
+          <t xml:space="preserve">    ├─ 荒原逃亡/未登记（Wasteland Fugitive） ──→ C.Y. 42 · 警署悬赏与黑市提取常见目标</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="7" t="inlineStr"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 酿造帮奴役酿民（Syndicate Bonded） ──→ C.Y. 42 · 园区卖身条款 · 出逃即警署悬赏</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>赏金猎人（The Hunter） ──→ C.Y. 30– · 名义猎人 · 实质击晕提取客户指定酿民威士忌</t>
-        </is>
-      </c>
+      <c r="A24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>缉拿手（The Hunter） ──→ C.Y. 30– · 警署登记承包商 · 实质击晕提取售黑市</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 名义职能（Cover Role） ──→ 公会委托 · 追捕/回收酿民</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">    ├─ 名义职能（Cover Role） ──→ 警署悬赏 · 抓捕凶犯与潜逃奴役酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">    └─ 实质产业链（Black Market Chain） ──→ 击晕→非法体内提取→黑市兑售</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
@@ -1156,6 +1181,7 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A9:C9"/>
@@ -1257,7 +1283,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 荒原模式（Wasteland Extraction） ──→ C.Y. 42 · 客户指定酿民 · 击晕提取 · 黑市出手</t>
+          <t xml:space="preserve">    ├─ 荒原模式（Wasteland Extraction） ──→ C.Y. 42 · 警署悬赏 · 击晕提取 · 黑市出手</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1318,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1352,28 +1378,380 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 荒原 The Wastes ──→ 城缘至铁瓶驿道 · 悬赏与提取</t>
+          <t xml:space="preserve">    └─ 荒原 The Wastes ──→ 城缘至铁瓶驿道 · 警署悬赏与提取</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ├─ 赏金猎人公会（Hunters Guild） ──→ 名义委托中介 · 锈钉接活</t>
+          <t xml:space="preserve">        ├─ 当地警署（Constabulary Post） ──→ 悬赏布告 · 登记缉拿手 · 锈钉接活</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">        ├─ 酿造帮园区（Brewing Syndicate） ──→ 高利贷奴役酿造 · 出逃悬赏</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">        └─ Saloon黑市链（Saloon Black Market） ──→ 回收槽收酵 · 威士忌出手</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 8. 势力格局</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>城酿署（Metro Brew Registry） ──→ C.Y. 42 · 酿民登记 · 采酿配额 · 禁猎保护</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>琥珀交易所（Amber Exchange） ──→ C.Y. 42 · 威士忌分级定价 · 货币</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>精品窖行（Vintage Vault Houses） ──→ C.Y. 42 · 签约精品酿民 · 暗中推动酿造帮收编脱约者</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>当地警署（Constabulary Post） ──→ C.Y. 42 · 悬赏缉拿 · 抓捕凶犯与潜逃奴役酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>酿造帮（Brewing Syndicate） ──→ C.Y. 42 · 高利贷园区 · 诓骗酿民卖身 · 非人权组织</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>铁瓶（生态群）（Synth-Rig Ecology） ──→ C.Y. 42 · 演化群落 · 一代酿民驻内 · 伴生未觉醒二代酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Saloon黑市链（Saloon Black Market） ──→ C.Y. 42 · 回收槽收酵 · 非法威士忌出手</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 与酿民敌对 · 完全摒弃/圣火 · 见8b</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避警署/酿造帮/戒酒教</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>漂沦者（The Wander） ──→ C.Y. 42 · 警署高危悬赏群体 · 锈钉禁忌</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A16:C16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 8a. 当地警署</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>当地警署（Constabulary Post） ──→ C.Y. 42 · 悬赏布告与接取 · 取代猎人公会</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 职能（Functions） ──→ 抓捕凶犯 · 追捕潜逃奴役酿民 · 羁押移交</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 悬赏四类（Bounty Categories） ──→ 酿民/圣火派/凶犯/漂沦者</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       ├─ 酿民类（Brewfolk Bounties） ──→ 出逃奴役酿民 · 脱约精品酿民 · 未登记者</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       ├─ 圣火派（Sacred Fire Bounties） ──→ 戒酒教净化武装 · 格杀勿论</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       ├─ 凶犯类（Felony Bounties） ──→ 谋杀犯 · 劫酵/劫火 · 袭警</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 漂沦者（Wander Bounties） ──→ 高危群体 · 活捉隔离/格杀许可</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 缉拿手制度（Contractor System） ──→ 登记接活 · 名义抓捕 · 实质黑市提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 驿站驻点（Outpost Posts） ──→ 城缘Saloon旁 · 锈钉挂牌处</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 8c. 酿造帮</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>酿造帮（Brewing Syndicate） ──→ C.Y. 42 · 高利贷奴役集团 · 非人权组织</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 诱贷（Debt Trap） ──→ 滤材酵苗医疗通行费 · 复利滚欠</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 卖身条款（Bondage Contract） ──→ 终身酿造义务 · 出逃全债加速 · 窖芯抵押</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 园区囚禁（Compound Yards） ──→ 围栏发酵舱 · 24垦时排班 · 编号管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 出逃悬赏（Escape Bounties） ──→ 向警署挂潜逃奴役酿民 · 园区出酬金</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 与窖行（Vault House Ties） ──→ 精品筛选转卖灰市 · 脱约者洗合同收编</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 对外形象（Public Face） ──→ 宣传安置就业 · 实际债务陷阱无退出</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
@@ -1387,127 +1765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与源》· 8. 势力格局</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>城酿署（Metro Brew Registry） ──→ C.Y. 42 · 酿民登记 · 采酿配额 · 禁猎保护</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>琥珀交易所（Amber Exchange） ──→ C.Y. 42 · 威士忌分级定价 · 货币</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>精品窖行（Vintage Vault Houses） ──→ C.Y. 42 · 签约精品酿民 · 暗中悬赏回收脱约者</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>铁瓶（生态群）（Synth-Rig Ecology） ──→ C.Y. 42 · 演化群落 · 一代酿民驻内 · 伴生未觉醒二代酿民</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>赏金猎人公会（Hunters Guild） ──→ C.Y. 42 · 名义委托中介 · 锈钉隶属</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Saloon黑市链（Saloon Black Market） ──→ C.Y. 42 · 回收槽收酵 · 非法威士忌出手</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 与酿民敌对 · 完全摒弃/圣火 · 见8b</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人与戒酒教</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="A15:C15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1582,7 +1840,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 隔离/诱捕移交/告密 · 不亲手焚杀</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 隔离/诱捕移交警署/告密 · 不亲手焚杀</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1854,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可付情报费借猎人刀</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可付情报费借缉拿手刀</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1929,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -1694,7 +1952,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 警署缉拿手 · 击晕提取售黑市 · 精品窖七破局</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1982,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
+          <t>酿造帮园区酿民（Syndicate Bonded Brewfolk） ──→ C.Y. 42 · 卖身条款 · 出逃悬赏 · R-xxx编号</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1992,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>戒酒教完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼 · 用泉不用窖 · 隔离诱捕酿民</t>
+          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
         </is>
       </c>
     </row>
@@ -1744,7 +2002,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>戒酒教圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼 · 秽须焚 · 焚杀酿民</t>
+          <t>戒酒教完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼 · 用泉不用窖 · 隔离诱捕酿民</t>
         </is>
       </c>
     </row>
@@ -1754,32 +2012,56 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>戒酒教圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼 · 秽须焚 · 警署悬赏目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>当地警署缉拿手（Constabulary Contractor） ──→ C.Y. 42 · 悬赏四类 · 锈钉式黑市提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
           <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="18">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A16:C16"/>
     <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1802,7 +2084,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
+          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义缉拿手 · 实质非法提取手 · 主线视角</t>
         </is>
       </c>
     </row>
@@ -1816,28 +2098,28 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
+          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 当地警署登记缉拿手 Constabulary Contractor</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
+          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接悬赏→击晕酿民目标→非法提取威士忌→黑市出手</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
+          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问悬赏背后 · 只关心酬金</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
+          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道警署驻点</t>
         </is>
       </c>
     </row>
@@ -1851,7 +2133,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
+          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不接漂沦者悬赏</t>
         </is>
       </c>
     </row>
@@ -1866,90 +2148,6 @@
   <mergeCells count="10">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与源》· 11. 锈钉开篇</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 非法提取链</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七提取委托 ×5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 背景侧写（Metro Contrast） ──→ 合法采酿行情 vs 黑市提取价</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
@@ -1969,7 +2167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C204"/>
+  <dimension ref="A1:C236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -2484,7 +2682,7 @@
     <row r="81" outlineLevel="1" ht="16" customHeight="1">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 赏金猎人（The Hunter） ──→ C.Y. 30– · 名义追捕 · 实质击晕提取售黑市</t>
+          <t xml:space="preserve">    └─ 缉拿手（The Hunter） ──→ C.Y. 30– · 警署悬赏承包商 · 实质击晕提取售黑市</t>
         </is>
       </c>
     </row>
@@ -2619,216 +2817,220 @@
     <row r="103" outlineLevel="1" ht="16" customHeight="1">
       <c r="A103" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 荒原逃亡/未登记（Wasteland Fugitive） ──→ C.Y. 42 · 脱离群落或从未登记 · 提取委托常见目标</t>
+          <t xml:space="preserve">    ├─ 荒原逃亡/未登记（Wasteland Fugitive） ──→ C.Y. 42 · 警署悬赏与黑市提取常见目标</t>
         </is>
       </c>
     </row>
     <row r="104" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A104" s="7" t="inlineStr"/>
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 酿造帮奴役酿民（Syndicate Bonded） ──→ C.Y. 42 · 园区卖身条款 · 出逃即警署悬赏</t>
+        </is>
+      </c>
     </row>
     <row r="105" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A105" s="7" t="inlineStr">
-        <is>
-          <t>赏金猎人（The Hunter） ──→ C.Y. 30– · 名义猎人 · 实质击晕提取客户指定酿民威士忌</t>
-        </is>
-      </c>
+      <c r="A105" s="7" t="inlineStr"/>
     </row>
     <row r="106" outlineLevel="1" ht="16" customHeight="1">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>缉拿手（The Hunter） ──→ C.Y. 30– · 警署登记承包商 · 实质击晕提取售黑市</t>
         </is>
       </c>
     </row>
     <row r="107" outlineLevel="1" ht="16" customHeight="1">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 名义职能（Cover Role） ──→ 公会委托 · 追捕/回收酿民</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="108" outlineLevel="1" ht="16" customHeight="1">
       <c r="A108" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">    ├─ 名义职能（Cover Role） ──→ 警署悬赏 · 抓捕凶犯与潜逃奴役酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">    └─ 实质产业链（Black Market Chain） ──→ 击晕→非法体内提取→黑市兑售</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="6" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="6" t="inlineStr">
         <is>
           <t>▸ 7. 威士忌经济</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A111" s="7" t="inlineStr">
-        <is>
-          <t>威士忌经济（Whiskey Economy） ──→ C.Y. 28– · 城带合法采酿 · 荒原非法提取黑市</t>
         </is>
       </c>
     </row>
     <row r="112" outlineLevel="1" ht="16" customHeight="1">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>威士忌经济（Whiskey Economy） ──→ C.Y. 28– · 城带合法采酿 · 荒原非法提取黑市</t>
         </is>
       </c>
     </row>
     <row r="113" outlineLevel="1" ht="16" customHeight="1">
       <c r="A113" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 原料（Input） ──→ 锈水（化学毒+嗜盐菌）</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="114" outlineLevel="1" ht="16" customHeight="1">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 转化（Fermentation） ──→ 酿民体内生态酵母 → 2–4%威士忌</t>
+          <t xml:space="preserve">    ├─ 原料（Input） ──→ 锈水（化学毒+嗜盐菌）</t>
         </is>
       </c>
     </row>
     <row r="115" outlineLevel="1" ht="16" customHeight="1">
       <c r="A115" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 品质分级（Quality Tiers） ──→ C.Y. 42 · 劣酿Row/常酿Standard/窖酿Vintage</t>
+          <t xml:space="preserve">    ├─ 转化（Fermentation） ──→ 酿民体内生态酵母 → 2–4%威士忌</t>
         </is>
       </c>
     </row>
     <row r="116" outlineLevel="1" ht="16" customHeight="1">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 劣酿 Row（Row Grade） ──→ 杂味重 · 荒原批量 · 猎人提取兑售</t>
+          <t xml:space="preserve">    ├─ 品质分级（Quality Tiers） ──→ C.Y. 42 · 劣酿Row/常酿Standard/窖酿Vintage</t>
         </is>
       </c>
     </row>
     <row r="117" outlineLevel="1" ht="16" customHeight="1">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 常酿 Standard（Standard Grade） ──→ 城带日常流通 · 登记酿民定期供酿</t>
+          <t xml:space="preserve">    │       ├─ 劣酿 Row（Row Grade） ──→ 杂味重 · 荒原批量 · 猎人提取兑售</t>
         </is>
       </c>
     </row>
     <row r="118" outlineLevel="1" ht="16" customHeight="1">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 窖酿 Vintage（Vintage Grade） ──→ 精品酿民专属 · 溢价极高</t>
+          <t xml:space="preserve">    │       ├─ 常酿 Standard（Standard Grade） ──→ 城带日常流通 · 登记酿民定期供酿</t>
         </is>
       </c>
     </row>
     <row r="119" outlineLevel="1" ht="16" customHeight="1">
       <c r="A119" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 城带模式（Metro Trade） ──→ C.Y. 42 · 登记采酿换琥珀币 · 琥珀交易所挂牌</t>
+          <t xml:space="preserve">    │       └─ 窖酿 Vintage（Vintage Grade） ──→ 精品酿民专属 · 溢价极高</t>
         </is>
       </c>
     </row>
     <row r="120" outlineLevel="1" ht="16" customHeight="1">
       <c r="A120" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 荒原模式（Wasteland Extraction） ──→ C.Y. 42 · 客户指定酿民 · 击晕提取 · 黑市出手</t>
+          <t xml:space="preserve">    ├─ 城带模式（Metro Trade） ──→ C.Y. 42 · 登记采酿换琥珀币 · 琥珀交易所挂牌</t>
         </is>
       </c>
     </row>
     <row r="121" outlineLevel="1" ht="16" customHeight="1">
       <c r="A121" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">    ├─ 荒原模式（Wasteland Extraction） ──→ C.Y. 42 · 警署悬赏 · 击晕提取 · 黑市出手</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">    └─ 裂缝（Fracture） ──→ C.Y. 37+ · 城带法规保护 vs 荒原无法无天</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="6" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="6" t="inlineStr">
         <is>
           <t>▸ 7b. 城带与荒原</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A124" s="7" t="inlineStr">
-        <is>
-          <t>城带与荒原（Metro Rim vs Wastes） ──→ C.Y. 42 · 赭锈带社会地理双态</t>
         </is>
       </c>
     </row>
     <row r="125" outlineLevel="1" ht="16" customHeight="1">
       <c r="A125" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>城带与荒原（Metro Rim vs Wastes） ──→ C.Y. 42 · 赭锈带社会地理双态</t>
         </is>
       </c>
     </row>
     <row r="126" outlineLevel="1" ht="16" customHeight="1">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 城带 Metro Rim ──→ 人类与二代酿民共存 · 非默认对立</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="127" outlineLevel="1" ht="16" customHeight="1">
       <c r="A127" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 城酿署（Metro Brew Registry） ──→ 登记 · 采酿配额 · 纠纷仲裁 · 禁猎保护</t>
+          <t xml:space="preserve">    ├─ 城带 Metro Rim ──→ 人类与二代酿民共存 · 非默认对立</t>
         </is>
       </c>
     </row>
     <row r="128" outlineLevel="1" ht="16" customHeight="1">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       ├─ 琥珀交易所（Amber Exchange） ──→ 威士忌品质挂牌 · 货币结算</t>
+          <t xml:space="preserve">    │       ├─ 城酿署（Metro Brew Registry） ──→ 登记 · 采酿配额 · 纠纷仲裁 · 禁猎保护</t>
         </is>
       </c>
     </row>
     <row r="129" outlineLevel="1" ht="16" customHeight="1">
       <c r="A129" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 精品窖行（Vintage Vault Houses） ──→ 竞签精品酿民 · 窖酿拍卖 · 暗中回收脱约者</t>
+          <t xml:space="preserve">    │       ├─ 琥珀交易所（Amber Exchange） ──→ 威士忌品质挂牌 · 货币结算</t>
         </is>
       </c>
     </row>
     <row r="130" outlineLevel="1" ht="16" customHeight="1">
       <c r="A130" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 荒原 The Wastes ──→ 城缘至铁瓶驿道 · 悬赏与提取</t>
+          <t xml:space="preserve">    │       └─ 精品窖行（Vintage Vault Houses） ──→ 竞签精品酿民 · 窖酿拍卖 · 暗中回收脱约者</t>
         </is>
       </c>
     </row>
     <row r="131" outlineLevel="1" ht="16" customHeight="1">
       <c r="A131" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">        ├─ 赏金猎人公会（Hunters Guild） ──→ 名义委托中介 · 锈钉接活</t>
+          <t xml:space="preserve">    └─ 荒原 The Wastes ──→ 城缘至铁瓶驿道 · 警署悬赏与提取</t>
         </is>
       </c>
     </row>
     <row r="132" outlineLevel="1" ht="16" customHeight="1">
       <c r="A132" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">        ├─ 当地警署（Constabulary Post） ──→ 悬赏布告 · 登记缉拿手 · 锈钉接活</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        ├─ 酿造帮园区（Brewing Syndicate） ──→ 高利贷奴役酿造 · 出逃悬赏</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">        └─ Saloon黑市链（Saloon Black Market） ──→ 回收槽收酵 · 威士忌出手</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="6" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="6" t="inlineStr">
         <is>
           <t>▸ 8. 势力格局</t>
         </is>
       </c>
-    </row>
-    <row r="135" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A135" s="7" t="inlineStr">
-        <is>
-          <t>城酿署（Metro Brew Registry） ──→ C.Y. 42 · 酿民登记 · 采酿配额 · 禁猎保护</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A136" s="7" t="inlineStr"/>
     </row>
     <row r="137" outlineLevel="1" ht="16" customHeight="1">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>琥珀交易所（Amber Exchange） ──→ C.Y. 42 · 威士忌分级定价 · 货币</t>
+          <t>城酿署（Metro Brew Registry） ──→ C.Y. 42 · 酿民登记 · 采酿配额 · 禁猎保护</t>
         </is>
       </c>
     </row>
@@ -2838,7 +3040,7 @@
     <row r="139" outlineLevel="1" ht="16" customHeight="1">
       <c r="A139" s="7" t="inlineStr">
         <is>
-          <t>精品窖行（Vintage Vault Houses） ──→ C.Y. 42 · 签约精品酿民 · 暗中悬赏回收脱约者</t>
+          <t>琥珀交易所（Amber Exchange） ──→ C.Y. 42 · 威士忌分级定价 · 货币</t>
         </is>
       </c>
     </row>
@@ -2848,7 +3050,7 @@
     <row r="141" outlineLevel="1" ht="16" customHeight="1">
       <c r="A141" s="7" t="inlineStr">
         <is>
-          <t>铁瓶（生态群）（Synth-Rig Ecology） ──→ C.Y. 42 · 演化群落 · 一代酿民驻内 · 伴生未觉醒二代酿民</t>
+          <t>精品窖行（Vintage Vault Houses） ──→ C.Y. 42 · 签约精品酿民 · 暗中推动酿造帮收编脱约者</t>
         </is>
       </c>
     </row>
@@ -2858,7 +3060,7 @@
     <row r="143" outlineLevel="1" ht="16" customHeight="1">
       <c r="A143" s="7" t="inlineStr">
         <is>
-          <t>赏金猎人公会（Hunters Guild） ──→ C.Y. 42 · 名义委托中介 · 锈钉隶属</t>
+          <t>当地警署（Constabulary Post） ──→ C.Y. 42 · 悬赏缉拿 · 抓捕凶犯与潜逃奴役酿民</t>
         </is>
       </c>
     </row>
@@ -2868,7 +3070,7 @@
     <row r="145" outlineLevel="1" ht="16" customHeight="1">
       <c r="A145" s="7" t="inlineStr">
         <is>
-          <t>Saloon黑市链（Saloon Black Market） ──→ C.Y. 42 · 回收槽收酵 · 非法威士忌出手</t>
+          <t>酿造帮（Brewing Syndicate） ──→ C.Y. 42 · 高利贷园区 · 诓骗酿民卖身 · 非人权组织</t>
         </is>
       </c>
     </row>
@@ -2878,7 +3080,7 @@
     <row r="147" outlineLevel="1" ht="16" customHeight="1">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 与酿民敌对 · 完全摒弃/圣火 · 见8b</t>
+          <t>铁瓶（生态群）（Synth-Rig Ecology） ──→ C.Y. 42 · 演化群落 · 一代酿民驻内 · 伴生未觉醒二代酿民</t>
         </is>
       </c>
     </row>
@@ -2888,343 +3090,535 @@
     <row r="149" outlineLevel="1" ht="16" customHeight="1">
       <c r="A149" s="7" t="inlineStr">
         <is>
-          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避猎人与戒酒教</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="6" t="inlineStr">
-        <is>
-          <t>▸ 8b. 戒酒教</t>
+          <t>Saloon黑市链（Saloon Black Market） ──→ C.Y. 42 · 回收槽收酵 · 非法威士忌出手</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A150" s="7" t="inlineStr"/>
+    </row>
+    <row r="151" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 与酿民敌对 · 完全摒弃/圣火 · 见8b</t>
         </is>
       </c>
     </row>
     <row r="152" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A152" s="7" t="inlineStr">
-        <is>
-          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 酿民即秽种 · 与酿民敌对 · 教团分裂</t>
-        </is>
-      </c>
+      <c r="A152" s="7" t="inlineStr"/>
     </row>
     <row r="153" outlineLevel="1" ht="16" customHeight="1">
       <c r="A153" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>逃亡酿民网络（Fugitive Brewfolk） ──→ C.Y. 42 · 未登记者互助 · 躲避警署/酿造帮/戒酒教</t>
         </is>
       </c>
     </row>
     <row r="154" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A154" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 共同教义（Shared Creed） ──→ 不庇护酿民 · 禁饮体内威士忌</t>
-        </is>
-      </c>
+      <c r="A154" s="7" t="inlineStr"/>
     </row>
     <row r="155" outlineLevel="1" ht="16" customHeight="1">
       <c r="A155" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿后 · 处置秽种路线之争</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A156" s="7" t="inlineStr"/>
-    </row>
-    <row r="157" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A157" s="7" t="inlineStr">
-        <is>
-          <t>完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼温和 · 用泉不用窖</t>
+          <t>漂沦者（The Wander） ──→ C.Y. 42 · 警署高危悬赏群体 · 锈钉禁忌</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>▸ 8a. 当地警署</t>
         </is>
       </c>
     </row>
     <row r="158" outlineLevel="1" ht="16" customHeight="1">
       <c r="A158" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t>当地警署（Constabulary Post） ──→ C.Y. 42 · 悬赏布告与接取 · 取代猎人公会</t>
         </is>
       </c>
     </row>
     <row r="159" outlineLevel="1" ht="16" customHeight="1">
       <c r="A159" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 利用离体酵母锈水 · 完全摒弃酿民</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="160" outlineLevel="1" ht="16" customHeight="1">
       <c r="A160" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 隔离/诱捕移交/告密 · 不亲手焚杀</t>
+          <t xml:space="preserve">    ├─ 职能（Functions） ──→ 抓捕凶犯 · 追捕潜逃奴役酿民 · 羁押移交</t>
         </is>
       </c>
     </row>
     <row r="161" outlineLevel="1" ht="16" customHeight="1">
       <c r="A161" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 净泉聚落（Pure Spring Communes） ──→ 离体培菌去毒 · 卖洁净锈水</t>
+          <t xml:space="preserve">    ├─ 悬赏四类（Bounty Categories） ──→ 酿民/圣火派/凶犯/漂沦者</t>
         </is>
       </c>
     </row>
     <row r="162" outlineLevel="1" ht="16" customHeight="1">
       <c r="A162" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可付情报费借猎人刀</t>
+          <t xml:space="preserve">    │       ├─ 酿民类（Brewfolk Bounties） ──→ 出逃奴役酿民 · 脱约精品酿民 · 未登记者</t>
         </is>
       </c>
     </row>
     <row r="163" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A163" s="7" t="inlineStr"/>
+      <c r="A163" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       ├─ 圣火派（Sacred Fire Bounties） ──→ 戒酒教净化武装 · 格杀勿论</t>
+        </is>
+      </c>
     </row>
     <row r="164" outlineLevel="1" ht="16" customHeight="1">
       <c r="A164" s="7" t="inlineStr">
         <is>
-          <t>圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼极端 · 秽须焚</t>
+          <t xml:space="preserve">    │       ├─ 凶犯类（Felony Bounties） ──→ 谋杀犯 · 劫酵/劫火 · 袭警</t>
         </is>
       </c>
     </row>
     <row r="165" outlineLevel="1" ht="16" customHeight="1">
       <c r="A165" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    │       └─ 漂沦者（Wander Bounties） ──→ 高危群体 · 活捉隔离/格杀许可</t>
         </is>
       </c>
     </row>
     <row r="166" outlineLevel="1" ht="16" customHeight="1">
       <c r="A166" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 酿民须圣火净化 · 不留窖芯</t>
+          <t xml:space="preserve">    ├─ 缉拿手制度（Contractor System） ──→ 登记接活 · 名义抓捕 · 实质黑市提取</t>
         </is>
       </c>
     </row>
     <row r="167" outlineLevel="1" ht="16" customHeight="1">
       <c r="A167" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 焚杀酿民/回收槽/铁瓶外露舱</t>
-        </is>
-      </c>
-    </row>
-    <row r="168" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A168" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 尘骑殉火（Dust Riders） ──→ 机动圣战 · 十三月尘暴掩护</t>
-        </is>
-      </c>
-    </row>
-    <row r="169" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A169" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 必杀 · 提取手与秽种同焚</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="6" t="inlineStr">
-        <is>
-          <t>▸ 9. 叙事入口</t>
+          <t xml:space="preserve">    └─ 驿站驻点（Outpost Posts） ──→ 城缘Saloon旁 · 锈钉挂牌处</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>▸ 8c. 酿造帮</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A170" s="7" t="inlineStr">
+        <is>
+          <t>酿造帮（Brewing Syndicate） ──→ C.Y. 42 · 高利贷奴役集团 · 非人权组织</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A171" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="172" outlineLevel="1" ht="16" customHeight="1">
       <c r="A172" s="7" t="inlineStr">
         <is>
-          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 名义猎人 · 击晕提取售黑市 · 精品窖七破局</t>
+          <t xml:space="preserve">    ├─ 诱贷（Debt Trap） ──→ 滤材酵苗医疗通行费 · 复利滚欠</t>
         </is>
       </c>
     </row>
     <row r="173" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A173" s="7" t="inlineStr"/>
+      <c r="A173" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 卖身条款（Bondage Contract） ──→ 终身酿造义务 · 出逃全债加速 · 窖芯抵押</t>
+        </is>
+      </c>
     </row>
     <row r="174" outlineLevel="1" ht="16" customHeight="1">
       <c r="A174" s="7" t="inlineStr">
         <is>
-          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
+          <t xml:space="preserve">    ├─ 园区囚禁（Compound Yards） ──→ 围栏发酵舱 · 24垦时排班 · 编号管理</t>
         </is>
       </c>
     </row>
     <row r="175" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A175" s="7" t="inlineStr"/>
+      <c r="A175" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 出逃悬赏（Escape Bounties） ──→ 向警署挂潜逃奴役酿民 · 园区出酬金</t>
+        </is>
+      </c>
     </row>
     <row r="176" outlineLevel="1" ht="16" customHeight="1">
       <c r="A176" s="7" t="inlineStr">
         <is>
-          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
+          <t xml:space="preserve">    ├─ 与窖行（Vault House Ties） ──→ 精品筛选转卖灰市 · 脱约者洗合同收编</t>
         </is>
       </c>
     </row>
     <row r="177" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A177" s="7" t="inlineStr"/>
-    </row>
-    <row r="178" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A178" s="7" t="inlineStr">
-        <is>
-          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
-        </is>
-      </c>
-    </row>
-    <row r="179" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A179" s="7" t="inlineStr"/>
+      <c r="A177" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 对外形象（Public Face） ──→ 宣传安置就业 · 实际债务陷阱无退出</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="6" t="inlineStr">
+        <is>
+          <t>▸ 8b. 戒酒教</t>
+        </is>
+      </c>
     </row>
     <row r="180" outlineLevel="1" ht="16" customHeight="1">
       <c r="A180" s="7" t="inlineStr">
         <is>
-          <t>戒酒教完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼 · 用泉不用窖 · 隔离诱捕酿民</t>
+          <t>戒酒教残存（Temperance Riders） ──→ C.Y. 42 · 酿民即秽种 · 与酿民敌对 · 教团分裂</t>
         </is>
       </c>
     </row>
     <row r="181" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A181" s="7" t="inlineStr"/>
+      <c r="A181" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
     </row>
     <row r="182" outlineLevel="1" ht="16" customHeight="1">
       <c r="A182" s="7" t="inlineStr">
         <is>
-          <t>戒酒教圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼 · 秽须焚 · 焚杀酿民</t>
+          <t xml:space="preserve">    ├─ 共同教义（Shared Creed） ──→ 不庇护酿民 · 禁饮体内威士忌</t>
         </is>
       </c>
     </row>
     <row r="183" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A183" s="7" t="inlineStr"/>
+      <c r="A183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 分裂契机（Schism） ──→ C.Y. 28–32 · 城带合法采酿后 · 处置秽种路线之争</t>
+        </is>
+      </c>
     </row>
     <row r="184" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A184" s="7" t="inlineStr">
-        <is>
-          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="6" t="inlineStr">
-        <is>
-          <t>▸ 10. 锈钉</t>
+      <c r="A184" s="7" t="inlineStr"/>
+    </row>
+    <row r="185" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A185" s="7" t="inlineStr">
+        <is>
+          <t>完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼温和 · 用泉不用窖</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A186" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="187" outlineLevel="1" ht="16" customHeight="1">
       <c r="A187" s="7" t="inlineStr">
         <is>
-          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义猎人 · 实质非法提取手 · 主线视角</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 利用离体酵母锈水 · 完全摒弃酿民</t>
         </is>
       </c>
     </row>
     <row r="188" outlineLevel="1" ht="16" customHeight="1">
       <c r="A188" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 隔离/诱捕移交警署/告密 · 不亲手焚杀</t>
         </is>
       </c>
     </row>
     <row r="189" outlineLevel="1" ht="16" customHeight="1">
       <c r="A189" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 赏金猎人公会登记手 The Hunter</t>
+          <t xml:space="preserve">    ├─ 净泉聚落（Pure Spring Communes） ──→ 离体培菌去毒 · 卖洁净锈水</t>
         </is>
       </c>
     </row>
     <row r="190" outlineLevel="1" ht="16" customHeight="1">
       <c r="A190" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接委托→击晕指定酿民→非法提取威士忌→黑市出手</t>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 可付情报费借缉拿手刀</t>
         </is>
       </c>
     </row>
     <row r="191" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A191" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问客户与目标 · 只关心酬金</t>
-        </is>
-      </c>
+      <c r="A191" s="7" t="inlineStr"/>
     </row>
     <row r="192" outlineLevel="1" ht="16" customHeight="1">
       <c r="A192" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道 · 不进城酿署体系</t>
+          <t>圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼极端 · 秽须焚</t>
         </is>
       </c>
     </row>
     <row r="193" outlineLevel="1" ht="16" customHeight="1">
       <c r="A193" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
+          <t xml:space="preserve">    │</t>
         </is>
       </c>
     </row>
     <row r="194" outlineLevel="1" ht="16" customHeight="1">
       <c r="A194" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不猎漂沦者</t>
+          <t xml:space="preserve">    ├─ 教义（Doctrine） ──→ 酿民须圣火净化 · 不留窖芯</t>
         </is>
       </c>
     </row>
     <row r="195" outlineLevel="1" ht="16" customHeight="1">
       <c r="A195" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" s="6" t="inlineStr">
-        <is>
-          <t>▸ 11. 锈钉开篇</t>
-        </is>
-      </c>
-    </row>
-    <row r="198" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A198" s="7" t="inlineStr">
-        <is>
-          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 非法提取链</t>
-        </is>
-      </c>
-    </row>
-    <row r="199" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A199" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
+          <t xml:space="preserve">    ├─ 手段（Methods） ──→ 焚杀酿民/回收槽/铁瓶外露舱</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 尘骑殉火（Dust Riders） ──→ 机动圣战 · 十三月尘暴掩护</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 对锈钉（On Rust Nail） ──→ 必杀 · 提取手与秽种同焚</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="6" t="inlineStr">
+        <is>
+          <t>▸ 9. 叙事入口</t>
         </is>
       </c>
     </row>
     <row r="200" outlineLevel="1" ht="16" customHeight="1">
       <c r="A200" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七提取委托 ×5</t>
+          <t>锈钉（Rust Nail） ──→ C.Y. 42 · 警署缉拿手 · 击晕提取售黑市 · 精品窖七破局</t>
         </is>
       </c>
     </row>
     <row r="201" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A201" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
-        </is>
-      </c>
+      <c r="A201" s="7" t="inlineStr"/>
     </row>
     <row r="202" outlineLevel="1" ht="16" customHeight="1">
       <c r="A202" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
+          <t>精品酿民窖七（Vintage Cellar-7） ──→ C.Y. 42 · 开篇对手 · 城带价码对峙</t>
         </is>
       </c>
     </row>
     <row r="203" outlineLevel="1" ht="16" customHeight="1">
-      <c r="A203" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
-        </is>
-      </c>
+      <c r="A203" s="7" t="inlineStr"/>
     </row>
     <row r="204" outlineLevel="1" ht="16" customHeight="1">
       <c r="A204" s="7" t="inlineStr">
         <is>
+          <t>城带登记酿民（Registered Metro Brewfolk） ──→ C.Y. 42 · 体内威士忌换币 · 共存日常</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A205" s="7" t="inlineStr"/>
+    </row>
+    <row r="206" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A206" s="7" t="inlineStr">
+        <is>
+          <t>酿造帮园区酿民（Syndicate Bonded Brewfolk） ──→ C.Y. 42 · 卖身条款 · 出逃悬赏 · R-xxx编号</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A207" s="7" t="inlineStr"/>
+    </row>
+    <row r="208" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A208" s="7" t="inlineStr">
+        <is>
+          <t>铁瓶伴生酿民（Bottle-Companion Brewfolk） ──→ C.Y. 42 · 未觉醒二代 · 记录同伴觉醒脱离群落</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A209" s="7" t="inlineStr"/>
+    </row>
+    <row r="210" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A210" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教完全摒弃派（Total Rejection） ──→ C.Y. 42 · 左翼 · 用泉不用窖 · 隔离诱捕酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A211" s="7" t="inlineStr"/>
+    </row>
+    <row r="212" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A212" s="7" t="inlineStr">
+        <is>
+          <t>戒酒教圣火派（Sacred Fire） ──→ C.Y. 42 · 右翼 · 秽须焚 · 警署悬赏目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A213" s="7" t="inlineStr"/>
+    </row>
+    <row r="214" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A214" s="7" t="inlineStr">
+        <is>
+          <t>当地警署缉拿手（Constabulary Contractor） ──→ C.Y. 42 · 悬赏四类 · 锈钉式黑市提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A215" s="7" t="inlineStr"/>
+    </row>
+    <row r="216" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A216" s="7" t="inlineStr">
+        <is>
+          <t>漂沦者接触者（Wander Witness） ──→ C.Y. 42 · 持有泄露文件残页</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="6" t="inlineStr">
+        <is>
+          <t>▸ 10. 锈钉</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A219" s="7" t="inlineStr">
+        <is>
+          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义缉拿手 · 实质非法提取手 · 主线视角</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 当地警署登记缉拿手 Constabulary Contractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接悬赏→击晕酿民目标→非法提取威士忌→黑市出手</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A223" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问悬赏背后 · 只关心酬金</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道警署驻点</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A225" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A226" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不接漂沦者悬赏</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="6" t="inlineStr">
+        <is>
+          <t>▸ 11. 锈钉开篇</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A230" s="7" t="inlineStr">
+        <is>
+          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 警署悬赏与非法提取链</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A232" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七悬赏 ×5</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A233" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A234" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" outlineLevel="1" ht="16" customHeight="1">
+      <c r="A236" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">    └─ 背景侧写（Metro Contrast） ──→ 合法采酿行情 vs 黑市提取价</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="188">
+  <mergeCells count="218">
     <mergeCell ref="A128:C128"/>
     <mergeCell ref="A193:C193"/>
     <mergeCell ref="A80:C80"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A208:C208"/>
     <mergeCell ref="A89:C89"/>
+    <mergeCell ref="A233:C233"/>
     <mergeCell ref="A136:C136"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A105:C105"/>
@@ -3232,41 +3626,48 @@
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A57:C57"/>
     <mergeCell ref="A113:C113"/>
+    <mergeCell ref="A210:C210"/>
     <mergeCell ref="A179:C179"/>
+    <mergeCell ref="A235:C235"/>
     <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A185:C185"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A194:C194"/>
+    <mergeCell ref="A234:C234"/>
     <mergeCell ref="A181:C181"/>
     <mergeCell ref="A91:C91"/>
     <mergeCell ref="A184:C184"/>
     <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A156:C156"/>
     <mergeCell ref="A171:C171"/>
     <mergeCell ref="A52:C52"/>
     <mergeCell ref="A165:C165"/>
     <mergeCell ref="A63:C63"/>
     <mergeCell ref="A155:C155"/>
     <mergeCell ref="A93:C93"/>
+    <mergeCell ref="A220:C220"/>
     <mergeCell ref="A173:C173"/>
+    <mergeCell ref="A229:C229"/>
     <mergeCell ref="A130:C130"/>
     <mergeCell ref="A77:C77"/>
     <mergeCell ref="A34:C34"/>
     <mergeCell ref="A83:C83"/>
     <mergeCell ref="A148:C148"/>
     <mergeCell ref="A157:C157"/>
+    <mergeCell ref="A222:C222"/>
     <mergeCell ref="A49:C49"/>
     <mergeCell ref="A138:C138"/>
     <mergeCell ref="A132:C132"/>
-    <mergeCell ref="A110:C110"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A119:C119"/>
     <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A196:C196"/>
     <mergeCell ref="A174:C174"/>
+    <mergeCell ref="A205:C205"/>
     <mergeCell ref="A183:C183"/>
     <mergeCell ref="A66:C66"/>
     <mergeCell ref="A118:C118"/>
     <mergeCell ref="A75:C75"/>
-    <mergeCell ref="A198:C198"/>
+    <mergeCell ref="A133:C133"/>
     <mergeCell ref="A120:C120"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="A12:C12"/>
@@ -3278,6 +3679,8 @@
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A159:C159"/>
     <mergeCell ref="A97:C97"/>
+    <mergeCell ref="A219:C219"/>
+    <mergeCell ref="A224:C224"/>
     <mergeCell ref="A106:C106"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A4:C4"/>
@@ -3287,20 +3690,23 @@
     <mergeCell ref="A96:C96"/>
     <mergeCell ref="A147:C147"/>
     <mergeCell ref="A121:C121"/>
+    <mergeCell ref="A209:C209"/>
     <mergeCell ref="A161:C161"/>
     <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A170:C170"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A31:C31"/>
     <mergeCell ref="A202:C202"/>
     <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A211:C211"/>
     <mergeCell ref="A67:C67"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A186:C186"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A201:C201"/>
     <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A226:C226"/>
     <mergeCell ref="A60:C60"/>
-    <mergeCell ref="A123:C123"/>
     <mergeCell ref="A197:C197"/>
     <mergeCell ref="A146:C146"/>
     <mergeCell ref="A124:C124"/>
@@ -3308,28 +3714,37 @@
     <mergeCell ref="A172:C172"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A187:C187"/>
+    <mergeCell ref="A212:C212"/>
     <mergeCell ref="A99:C99"/>
     <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A221:C221"/>
     <mergeCell ref="A108:C108"/>
     <mergeCell ref="A84:C84"/>
+    <mergeCell ref="A236:C236"/>
     <mergeCell ref="A149:C149"/>
+    <mergeCell ref="A214:C214"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A163:C163"/>
     <mergeCell ref="A158:C158"/>
     <mergeCell ref="A101:C101"/>
     <mergeCell ref="A189:C189"/>
+    <mergeCell ref="A223:C223"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A86:C86"/>
     <mergeCell ref="A204:C204"/>
     <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A213:C213"/>
     <mergeCell ref="A151:C151"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A188:C188"/>
     <mergeCell ref="A126:C126"/>
     <mergeCell ref="A141:C141"/>
-    <mergeCell ref="A135:C135"/>
+    <mergeCell ref="A150:C150"/>
+    <mergeCell ref="A206:C206"/>
     <mergeCell ref="A62:C62"/>
     <mergeCell ref="A144:C144"/>
+    <mergeCell ref="A122:C122"/>
+    <mergeCell ref="A215:C215"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A125:C125"/>
     <mergeCell ref="A190:C190"/>
@@ -3350,13 +3765,14 @@
     <mergeCell ref="A98:C98"/>
     <mergeCell ref="A191:C191"/>
     <mergeCell ref="A169:C169"/>
+    <mergeCell ref="A225:C225"/>
     <mergeCell ref="A107:C107"/>
-    <mergeCell ref="A178:C178"/>
     <mergeCell ref="A79:C79"/>
     <mergeCell ref="A88:C88"/>
     <mergeCell ref="A70:C70"/>
     <mergeCell ref="A153:C153"/>
     <mergeCell ref="A162:C162"/>
+    <mergeCell ref="A227:C227"/>
     <mergeCell ref="A54:C54"/>
     <mergeCell ref="A137:C137"/>
     <mergeCell ref="A177:C177"/>
@@ -3382,13 +3798,16 @@
     <mergeCell ref="A100:C100"/>
     <mergeCell ref="A140:C140"/>
     <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A109:C109"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A180:C180"/>
+    <mergeCell ref="A231:C231"/>
     <mergeCell ref="A115:C115"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A68:C68"/>
     <mergeCell ref="A102:C102"/>
     <mergeCell ref="A117:C117"/>
+    <mergeCell ref="A230:C230"/>
     <mergeCell ref="A111:C111"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A143:C143"/>
@@ -3396,17 +3815,104 @@
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="A166:C166"/>
     <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A232:C232"/>
     <mergeCell ref="A142:C142"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A207:C207"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A94:C94"/>
     <mergeCell ref="A103:C103"/>
-    <mergeCell ref="A168:C168"/>
+    <mergeCell ref="A216:C216"/>
     <mergeCell ref="A78:C78"/>
     <mergeCell ref="A87:C87"/>
     <mergeCell ref="A65:C65"/>
+    <mergeCell ref="A218:C218"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 11. 锈钉开篇</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>开篇：行尸走肉（Opening: Zombie Loop） ──→ C.Y. 42 · 锈钉视角三幕 · 警署悬赏与非法提取链</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第一幕 接单（Act 1 Contract） ──→ Saloon · 交酵入回收槽 · 红标精品窖七悬赏 ×5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第二幕 追踪（Act 2 Trail） ──→ 驿道 · 接近击晕窗口 · 目标懂荒原</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 第三幕 照面（Act 3 Standoff） ──→ 水窖 · 城带窖酿行开价多少 · 黑市算术失灵</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 对手窖七（Target Cellar-7） ──→ 精品酿民 · 拒被击晕提取 · 交易语言</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 背景侧写（Metro Contrast） ──→ 合法采酿行情 vs 黑市提取价</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync BD docs 2026-07-08-v1 (202607200728) from my-cloud-project@553e9a7
</commit_message>
<xml_diff>
--- a/瓶与井世界观树状图.xlsx
+++ b/瓶与井世界观树状图.xlsx
@@ -9,24 +9,25 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部树状图" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0. 叙事边界" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. 赭锈带" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. 锈水" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. 十三月" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. 生态酵母" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5a. 第一批移民" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5b. 第二批移民" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5c. 第三批移民" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. 存在体谱系" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. 威士忌经济" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7b. 城带与荒原" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. 势力格局" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8a. 当地警署" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8c. 酿造帮" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. 戒酒教" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. 叙事入口" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. 锈钉" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 锈钉开篇" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="派系态度矩阵" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0. 叙事边界" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. 赭锈带" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. 锈水" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. 十三月" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. 生态酵母" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5a. 第一批移民" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5b. 第二批移民" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5c. 第三批移民" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. 存在体谱系" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. 威士忌经济" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7b. 城带与荒原" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. 势力格局" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8a. 当地警署" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8c. 酿造帮" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. 戒酒教" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. 叙事入口" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. 锈钉" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. 锈钉开篇" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +73,21 @@
       <color rgb="001F4E79"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -85,8 +99,28 @@
         <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005C4033"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8F9F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -94,11 +128,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4B4B4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +158,25 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -499,7 +566,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-07-20-v17</t>
+          <t>2026-07-20-v18</t>
         </is>
       </c>
     </row>
@@ -898,6 +965,114 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 5b. 第二批移民</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>第二批移民（Wave 2 Androids） ──→ C.Y. 8–25 · Android拓荒 · 真正一代酿民</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 一代酿民 Gen-1（Gen-1 Brewfolk） ──→ C.Y. 8–25 · 植入生态酵母的Android移民</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 铁瓶 Synth-Rig ──→ C.Y. 10– · Neo-Western行驶的地表改造酿运载具</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │   │</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 驻瓶（Bottle-Dwelling） ──→ C.Y. 10– · 一代酿民驻留铁瓶内改造荒原</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 二代酿民 Gen-2（Gen-2 Brewfolk） ──→ C.Y. 15– · 伴生铁瓶 · 分未觉醒伴生/觉醒迁出/城带登记</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │   │</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │       └─ 铁瓶伴生未觉醒（Bottle-Companion Gen-2） ──→ C.Y. 15– · 维护铁瓶生态群 · 多数无自主意识</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 觉醒迁出（Awakening Exodus） ──→ C.Y. 30+ · 自主意识 · 拒绝作酵母容器 · 逃亡</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -977,7 +1152,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1197,7 +1372,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1313,7 +1488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1421,7 +1596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1565,7 +1740,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1673,7 +1848,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1765,7 +1940,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1929,7 +2104,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2056,106 +2231,6 @@
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A15:C15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与源》· 10. 锈钉</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义缉拿手 · 实质非法提取手 · 主线视角</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 当地警署登记缉拿手 Constabulary Contractor</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接悬赏→击晕酿民目标→非法提取威士忌→黑市出手</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问悬赏背后 · 只关心酬金</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道警署驻点</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不接漂沦者悬赏</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3839,6 +3914,106 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="96" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 10. 锈钉</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>锈钉 Rust Nail ──→ C.Y. 42 · 名义缉拿手 · 实质非法提取手 · 主线视角</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    │</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 对外身份（Cover Identity） ──→ 当地警署登记缉拿手 Constabulary Contractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 实际工作（Actual Work） ──→ 接悬赏→击晕酿民目标→非法提取威士忌→黑市出手</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 状态（State） ──→ 开篇 · 行尸走肉 · 不追问悬赏背后 · 只关心酬金</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 活动区（Range） ──→ 城带外荒原/Saloon/驿道警署驻点</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 标志（Trait） ──→ 左腕锈迹酵管提取器 · 击晕与提取兼用</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ├─ 禁忌（Taboo） ──→ 不接漂沦者悬赏</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    └─ 第一裂隙（First Crack） ──→ Undecimber · 窖七用城带挂牌价逼他算账 · 击晕前停顿</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3922,6 +4097,1748 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>《瓶与源》· 派系态度矩阵（行 → 列）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>读法：行势力对列势力的态度 · v18 · 含组织派系与酿民群体</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>行＼列</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>城酿署
+(Metro Brew Registry)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>琥珀交易所
+(Amber Exchange)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>精品窖行
+(Vintage Vault Houses)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>当地警署
+(Constabulary Post)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>酿造帮
+(Brewing Syndicate)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>铁瓶生态群
+(Synth-Rig Ecology)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Saloon黑市链
+(Saloon Black Market)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>戒酒教·摒弃派
+(Total Rejection)</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>戒酒教·圣火派
+(Sacred Fire)</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>逃亡酿民网络
+(Fugitive Network)</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>漂沦者
+(The Wander)</t>
+        </is>
+      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>锈钉
+(Rust Nail)</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="inlineStr">
+        <is>
+          <t>城带登记酿民
+(Registered Metro Brewfolk)</t>
+        </is>
+      </c>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>园区奴役酿民
+(Syndicate Bonded Brewfolk)</t>
+        </is>
+      </c>
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>精品酿民
+(Vintage Brewfolk)</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>铁瓶伴生酿民
+(Bottle-Companion Brewfolk)</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr">
+        <is>
+          <t>逃亡/未登记酿民
+(Fugitive Brewfolk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>城酿署
+(Metro Brew Registry)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>合作</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>监管容忍</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>合作</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>疏远</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>疏远</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="L5" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>保护</t>
+        </is>
+      </c>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>不认可</t>
+        </is>
+      </c>
+      <c r="P5" s="12" t="inlineStr">
+        <is>
+          <t>保护</t>
+        </is>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="R5" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>琥珀交易所
+(Amber Exchange)</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>依赖</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>防备</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="N6" s="13" t="inlineStr">
+        <is>
+          <t>商品化</t>
+        </is>
+      </c>
+      <c r="O6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t>精品挂牌</t>
+        </is>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="R6" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>精品窖行
+(Vintage Vault Houses)</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>依赖</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>防备</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="N7" s="12" t="inlineStr">
+        <is>
+          <t>签约资产</t>
+        </is>
+      </c>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>收编来源</t>
+        </is>
+      </c>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>垄断目标</t>
+        </is>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>猎取潜力</t>
+        </is>
+      </c>
+      <c r="R7" s="14" t="inlineStr">
+        <is>
+          <t>追捕脱约</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>当地警署
+(Constabulary Post)</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>合作</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>容忍</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>合作</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>容忍</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>容忍</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="N8" s="12" t="inlineStr">
+        <is>
+          <t>保护</t>
+        </is>
+      </c>
+      <c r="O8" s="14" t="inlineStr">
+        <is>
+          <t>追捕出逃</t>
+        </is>
+      </c>
+      <c r="P8" s="14" t="inlineStr">
+        <is>
+          <t>追捕脱约</t>
+        </is>
+      </c>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="R8" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>酿造帮
+(Brewing Syndicate)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>追捕</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="N9" s="13" t="inlineStr">
+        <is>
+          <t>诱贷目标</t>
+        </is>
+      </c>
+      <c r="O9" s="13" t="inlineStr">
+        <is>
+          <t>工具化</t>
+        </is>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>转卖窖行</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>诱拐目标</t>
+        </is>
+      </c>
+      <c r="R9" s="14" t="inlineStr">
+        <is>
+          <t>追捕债奴</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>铁瓶生态群
+(Synth-Rig Ecology)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>疏远</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>疏远</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>防备</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>被抵制</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>被敌对</t>
+        </is>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>庇护</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>容忍</t>
+        </is>
+      </c>
+      <c r="N10" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="O10" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>觉醒可脱离</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>维护群落</t>
+        </is>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
+          <t>庇护迁出</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Saloon黑市链
+(Saloon Black Market)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>应付</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>被抵制</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>被敌对</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>容忍</t>
+        </is>
+      </c>
+      <c r="L11" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>酵源</t>
+        </is>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t>高价酵源</t>
+        </is>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="R11" s="13" t="inlineStr">
+        <is>
+          <t>酵源</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>戒酒教·摒弃派
+(Total Rejection)</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>抵制</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>抵制</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>抵制</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="N12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="O12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="P12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="Q12" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="R12" s="14" t="inlineStr">
+        <is>
+          <t>敌对·诱捕</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>戒酒教·圣火派
+(Sacred Fire)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="M13" s="14" t="inlineStr">
+        <is>
+          <t>必杀</t>
+        </is>
+      </c>
+      <c r="N13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="O13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="P13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="Q13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+      <c r="R13" s="14" t="inlineStr">
+        <is>
+          <t>焚杀</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>逃亡酿民网络
+(Fugitive Network)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>求助</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>互助</t>
+        </is>
+      </c>
+      <c r="L14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="M14" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>渴望</t>
+        </is>
+      </c>
+      <c r="O14" s="12" t="inlineStr">
+        <is>
+          <t>互助</t>
+        </is>
+      </c>
+      <c r="P14" s="12" t="inlineStr">
+        <is>
+          <t>互助</t>
+        </is>
+      </c>
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>互助</t>
+        </is>
+      </c>
+      <c r="R14" s="12" t="inlineStr">
+        <is>
+          <t>互助</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>漂沦者
+(The Wander)</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>被悬赏</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="R15" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>锈钉
+(Rust Nail)</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>无视</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>依赖</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>利用</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>依赖</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>疏远</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="inlineStr">
+        <is>
+          <t>禁忌</t>
+        </is>
+      </c>
+      <c r="M16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>提取目标</t>
+        </is>
+      </c>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>提取目标</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>一般不碰</t>
+        </is>
+      </c>
+      <c r="R16" s="13" t="inlineStr">
+        <is>
+          <t>提取目标</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>城带登记酿民
+(Registered Metro Brewfolk)</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>依赖</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>交易</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>被签约</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>受保护</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>警惕</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>被敌对</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>被焚杀</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="N17" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>对立</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>同类</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>同类</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t>对立</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>园区奴役酿民
+(Syndicate Bonded Brewfolk)</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>躲避</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>被转卖</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>被囚禁</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>被提取</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>被敌对</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="inlineStr">
+        <is>
+          <t>被焚杀</t>
+        </is>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>被互助</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>被提取</t>
+        </is>
+      </c>
+      <c r="N18" s="13" t="inlineStr">
+        <is>
+          <t>渴望逃离</t>
+        </is>
+      </c>
+      <c r="O18" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t>被筛选</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t>同类</t>
+        </is>
+      </c>
+      <c r="R18" s="13" t="inlineStr">
+        <is>
+          <t>逃亡同类</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>精品酿民
+(Vintage Brewfolk)</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>依赖/脱约</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>高价挂牌</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>被垄断</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>脱约被追捕</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>被转卖</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>可觉醒脱离</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>高价酵源</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t>被敌对</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>被焚杀</t>
+        </is>
+      </c>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>被庇护</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>高价目标</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>上位同类</t>
+        </is>
+      </c>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>逃出身份</t>
+        </is>
+      </c>
+      <c r="P19" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>潜在觉醒</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
+        <is>
+          <t>脱约同类</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>铁瓶伴生酿民
+(Bottle-Companion Brewfolk)</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>被猎取</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>被诱拐</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>依附群落</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="inlineStr">
+        <is>
+          <t>被敌对</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="inlineStr">
+        <is>
+          <t>被焚杀</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>觉醒可入</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>一般不碰</t>
+        </is>
+      </c>
+      <c r="N20" s="13" t="inlineStr">
+        <is>
+          <t>觉醒可入城</t>
+        </is>
+      </c>
+      <c r="O20" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>被筛选</t>
+        </is>
+      </c>
+      <c r="Q20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R20" s="13" t="inlineStr">
+        <is>
+          <t>觉醒迁出</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>逃亡/未登记酿民
+(Fugitive Brewfolk)</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>无关</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>被追捕</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>可获庇护</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>被提取</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>被诱捕</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>被焚杀</t>
+        </is>
+      </c>
+      <c r="K21" s="12" t="inlineStr">
+        <is>
+          <t>被互助</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>回避</t>
+        </is>
+      </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>被提取</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="inlineStr">
+        <is>
+          <t>渴望成为</t>
+        </is>
+      </c>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>逃出同类</t>
+        </is>
+      </c>
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t>脱约同类</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>迁出同类</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3986,7 +5903,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4094,7 +6011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4186,7 +6103,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4262,7 +6179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4341,106 +6258,6 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>《瓶与源》· 5a. 第一批移民</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>第一批移民（Wave 1 Humans） ──→ C.Y. 0–8 · 国家资源竞赛 · 胃植入生态酵母</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 背景（Context） ──→ C.Y. 0–8 · 多国争夺赭锈带</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 手段（Method） ──→ C.Y. 0–8 · 生态酵母植入首批移民胃中</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 真相泄露（Leak） ──→ C.Y. 5+ · 嗜盐菌0.05%存活率 · 神经毒素累积</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ├─ 畸变（Aberration） ──→ C.Y. 5–8 · 精神畸变+辐射尘 → 漂沦者</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │   │</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    │       └─ 漂沦者 The Wander ──→ C.Y. 8+ · 特殊生物磁场 · 尘暴游荡</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 结局（Outcome） ──→ C.Y. 8 · 国家撤回编制 · 人类移民失败</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
@@ -4459,7 +6276,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="96" customWidth="1" min="1" max="1"/>
@@ -4470,14 +6287,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>《瓶与源》· 5b. 第二批移民</t>
+          <t>《瓶与源》· 5a. 第一批移民</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>第二批移民（Wave 2 Androids） ──→ C.Y. 8–25 · Android拓荒 · 真正一代酿民</t>
+          <t>第一批移民（Wave 1 Humans） ──→ C.Y. 0–8 · 国家资源竞赛 · 胃植入生态酵母</t>
         </is>
       </c>
     </row>
@@ -4491,61 +6308,54 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 一代酿民 Gen-1（Gen-1 Brewfolk） ──→ C.Y. 8–25 · 植入生态酵母的Android移民</t>
+          <t xml:space="preserve">    ├─ 背景（Context） ──→ C.Y. 0–8 · 多国争夺赭锈带</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 铁瓶 Synth-Rig ──→ C.Y. 10– · Neo-Western行驶的地表改造酿运载具</t>
+          <t xml:space="preserve">    ├─ 手段（Method） ──→ C.Y. 0–8 · 生态酵母植入首批移民胃中</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │   │</t>
+          <t xml:space="preserve">    ├─ 真相泄露（Leak） ──→ C.Y. 5+ · 嗜盐菌0.05%存活率 · 神经毒素累积</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 驻瓶（Bottle-Dwelling） ──→ C.Y. 10– · 一代酿民驻留铁瓶内改造荒原</t>
+          <t xml:space="preserve">    ├─ 畸变（Aberration） ──→ C.Y. 5–8 · 精神畸变+辐射尘 → 漂沦者</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ├─ 二代酿民 Gen-2（Gen-2 Brewfolk） ──→ C.Y. 15– · 伴生铁瓶 · 分未觉醒伴生/觉醒迁出/城带登记</t>
+          <t xml:space="preserve">    │   │</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │   │</t>
+          <t xml:space="preserve">    │       └─ 漂沦者 The Wander ──→ C.Y. 8+ · 特殊生物磁场 · 尘暴游荡</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    │       └─ 铁瓶伴生未觉醒（Bottle-Companion Gen-2） ──→ C.Y. 15– · 维护铁瓶生态群 · 多数无自主意识</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    └─ 觉醒迁出（Awakening Exodus） ──→ C.Y. 30+ · 自主意识 · 拒绝作酵母容器 · 逃亡</t>
+          <t xml:space="preserve">    └─ 结局（Outcome） ──→ C.Y. 8 · 国家撤回编制 · 人类移民失败</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="10">
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
@@ -4555,7 +6365,6 @@
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>